<commit_message>
Daily price pull 2026-09-13
</commit_message>
<xml_diff>
--- a/tesla_price_analysis.xlsx
+++ b/tesla_price_analysis.xlsx
@@ -445,7 +445,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Snapshot date: 2026-09-12  (source: tesla.com configurator pages)</t>
+          <t>Snapshot date: 2026-09-13  (source: tesla.com configurator pages)</t>
         </is>
       </c>
       <c r="B1" s="1" t="n"/>
@@ -775,7 +775,7 @@
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="19" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -859,7 +859,7 @@
         <v>301125</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>303840</v>
+        <v>304827.2727272727</v>
       </c>
     </row>
   </sheetData>
@@ -971,7 +971,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G411"/>
+  <dimension ref="A1:G420"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -15370,6 +15370,321 @@
         </is>
       </c>
     </row>
+    <row r="412">
+      <c r="A412" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B412" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C412" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D412" s="2" t="inlineStr">
+        <is>
+          <t>MT373</t>
+        </is>
+      </c>
+      <c r="E412" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F412" s="3" t="n">
+        <v>235500</v>
+      </c>
+      <c r="G412" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B413" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C413" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D413" s="2" t="inlineStr">
+        <is>
+          <t>MT374</t>
+        </is>
+      </c>
+      <c r="E413" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F413" s="3" t="n">
+        <v>259500</v>
+      </c>
+      <c r="G413" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B414" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C414" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D414" s="2" t="inlineStr">
+        <is>
+          <t>MT375</t>
+        </is>
+      </c>
+      <c r="E414" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F414" s="3" t="n">
+        <v>285500</v>
+      </c>
+      <c r="G414" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B415" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C415" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D415" s="2" t="inlineStr">
+        <is>
+          <t>MT376</t>
+        </is>
+      </c>
+      <c r="E415" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F415" s="3" t="n">
+        <v>339500</v>
+      </c>
+      <c r="G415" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B416" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C416" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D416" s="2" t="inlineStr">
+        <is>
+          <t>MTY69</t>
+        </is>
+      </c>
+      <c r="E416" s="2" t="inlineStr">
+        <is>
+          <t>Model Y L</t>
+        </is>
+      </c>
+      <c r="F416" s="3" t="n">
+        <v>339000</v>
+      </c>
+      <c r="G416" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B417" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C417" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D417" s="2" t="inlineStr">
+        <is>
+          <t>MTY79</t>
+        </is>
+      </c>
+      <c r="E417" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F417" s="3" t="n">
+        <v>263500</v>
+      </c>
+      <c r="G417" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B418" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C418" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D418" s="2" t="inlineStr">
+        <is>
+          <t>MTY80</t>
+        </is>
+      </c>
+      <c r="E418" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F418" s="3" t="n">
+        <v>313500</v>
+      </c>
+      <c r="G418" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B419" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C419" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D419" s="2" t="inlineStr">
+        <is>
+          <t>MTY81</t>
+        </is>
+      </c>
+      <c r="E419" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F419" s="3" t="n">
+        <v>288500</v>
+      </c>
+      <c r="G419" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B420" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C420" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D420" s="2" t="inlineStr">
+        <is>
+          <t>MTY88</t>
+        </is>
+      </c>
+      <c r="E420" s="2" t="inlineStr">
+        <is>
+          <t>Model Y Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F420" s="3" t="n">
+        <v>369000</v>
+      </c>
+      <c r="G420" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price pull 2026-09-14
</commit_message>
<xml_diff>
--- a/tesla_price_analysis.xlsx
+++ b/tesla_price_analysis.xlsx
@@ -445,7 +445,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Snapshot date: 2026-09-13  (source: tesla.com configurator pages)</t>
+          <t>Snapshot date: 2026-09-14  (source: tesla.com configurator pages)</t>
         </is>
       </c>
       <c r="B1" s="1" t="n"/>
@@ -775,7 +775,7 @@
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="19" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -859,7 +859,7 @@
         <v>301125</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>304827.2727272727</v>
+        <v>305650</v>
       </c>
     </row>
   </sheetData>
@@ -971,7 +971,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G420"/>
+  <dimension ref="A1:G429"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -15685,6 +15685,321 @@
         </is>
       </c>
     </row>
+    <row r="421">
+      <c r="A421" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B421" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C421" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D421" s="2" t="inlineStr">
+        <is>
+          <t>MT373</t>
+        </is>
+      </c>
+      <c r="E421" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F421" s="3" t="n">
+        <v>235500</v>
+      </c>
+      <c r="G421" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B422" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C422" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D422" s="2" t="inlineStr">
+        <is>
+          <t>MT374</t>
+        </is>
+      </c>
+      <c r="E422" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F422" s="3" t="n">
+        <v>259500</v>
+      </c>
+      <c r="G422" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B423" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C423" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D423" s="2" t="inlineStr">
+        <is>
+          <t>MT375</t>
+        </is>
+      </c>
+      <c r="E423" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F423" s="3" t="n">
+        <v>285500</v>
+      </c>
+      <c r="G423" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B424" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C424" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D424" s="2" t="inlineStr">
+        <is>
+          <t>MT376</t>
+        </is>
+      </c>
+      <c r="E424" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F424" s="3" t="n">
+        <v>339500</v>
+      </c>
+      <c r="G424" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B425" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C425" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D425" s="2" t="inlineStr">
+        <is>
+          <t>MTY69</t>
+        </is>
+      </c>
+      <c r="E425" s="2" t="inlineStr">
+        <is>
+          <t>Model Y L</t>
+        </is>
+      </c>
+      <c r="F425" s="3" t="n">
+        <v>339000</v>
+      </c>
+      <c r="G425" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B426" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C426" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D426" s="2" t="inlineStr">
+        <is>
+          <t>MTY79</t>
+        </is>
+      </c>
+      <c r="E426" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F426" s="3" t="n">
+        <v>263500</v>
+      </c>
+      <c r="G426" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B427" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C427" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D427" s="2" t="inlineStr">
+        <is>
+          <t>MTY80</t>
+        </is>
+      </c>
+      <c r="E427" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F427" s="3" t="n">
+        <v>313500</v>
+      </c>
+      <c r="G427" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B428" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C428" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D428" s="2" t="inlineStr">
+        <is>
+          <t>MTY81</t>
+        </is>
+      </c>
+      <c r="E428" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F428" s="3" t="n">
+        <v>288500</v>
+      </c>
+      <c r="G428" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B429" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C429" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D429" s="2" t="inlineStr">
+        <is>
+          <t>MTY88</t>
+        </is>
+      </c>
+      <c r="E429" s="2" t="inlineStr">
+        <is>
+          <t>Model Y Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F429" s="3" t="n">
+        <v>369000</v>
+      </c>
+      <c r="G429" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price pull 2026-09-15
</commit_message>
<xml_diff>
--- a/tesla_price_analysis.xlsx
+++ b/tesla_price_analysis.xlsx
@@ -445,7 +445,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Snapshot date: 2026-09-14  (source: tesla.com configurator pages)</t>
+          <t>Snapshot date: 2026-09-15  (source: tesla.com configurator pages)</t>
         </is>
       </c>
       <c r="B1" s="1" t="n"/>
@@ -775,7 +775,7 @@
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="19" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -859,7 +859,7 @@
         <v>301125</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>305650</v>
+        <v>306346.1538461539</v>
       </c>
     </row>
   </sheetData>
@@ -971,7 +971,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G429"/>
+  <dimension ref="A1:G438"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -16000,6 +16000,321 @@
         </is>
       </c>
     </row>
+    <row r="430">
+      <c r="A430" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B430" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C430" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D430" s="2" t="inlineStr">
+        <is>
+          <t>MT373</t>
+        </is>
+      </c>
+      <c r="E430" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F430" s="3" t="n">
+        <v>235500</v>
+      </c>
+      <c r="G430" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B431" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C431" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D431" s="2" t="inlineStr">
+        <is>
+          <t>MT374</t>
+        </is>
+      </c>
+      <c r="E431" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F431" s="3" t="n">
+        <v>259500</v>
+      </c>
+      <c r="G431" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B432" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C432" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D432" s="2" t="inlineStr">
+        <is>
+          <t>MT375</t>
+        </is>
+      </c>
+      <c r="E432" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F432" s="3" t="n">
+        <v>285500</v>
+      </c>
+      <c r="G432" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B433" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C433" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D433" s="2" t="inlineStr">
+        <is>
+          <t>MT376</t>
+        </is>
+      </c>
+      <c r="E433" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F433" s="3" t="n">
+        <v>339500</v>
+      </c>
+      <c r="G433" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B434" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C434" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D434" s="2" t="inlineStr">
+        <is>
+          <t>MTY69</t>
+        </is>
+      </c>
+      <c r="E434" s="2" t="inlineStr">
+        <is>
+          <t>Model Y L</t>
+        </is>
+      </c>
+      <c r="F434" s="3" t="n">
+        <v>339000</v>
+      </c>
+      <c r="G434" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B435" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C435" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D435" s="2" t="inlineStr">
+        <is>
+          <t>MTY79</t>
+        </is>
+      </c>
+      <c r="E435" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F435" s="3" t="n">
+        <v>263500</v>
+      </c>
+      <c r="G435" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B436" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C436" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D436" s="2" t="inlineStr">
+        <is>
+          <t>MTY80</t>
+        </is>
+      </c>
+      <c r="E436" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F436" s="3" t="n">
+        <v>313500</v>
+      </c>
+      <c r="G436" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B437" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C437" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D437" s="2" t="inlineStr">
+        <is>
+          <t>MTY81</t>
+        </is>
+      </c>
+      <c r="E437" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F437" s="3" t="n">
+        <v>288500</v>
+      </c>
+      <c r="G437" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B438" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C438" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D438" s="2" t="inlineStr">
+        <is>
+          <t>MTY88</t>
+        </is>
+      </c>
+      <c r="E438" s="2" t="inlineStr">
+        <is>
+          <t>Model Y Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F438" s="3" t="n">
+        <v>369000</v>
+      </c>
+      <c r="G438" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price pull 2026-09-16
</commit_message>
<xml_diff>
--- a/tesla_price_analysis.xlsx
+++ b/tesla_price_analysis.xlsx
@@ -445,7 +445,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Snapshot date: 2026-09-15  (source: tesla.com configurator pages)</t>
+          <t>Snapshot date: 2026-09-16  (source: tesla.com configurator pages)</t>
         </is>
       </c>
       <c r="B1" s="1" t="n"/>
@@ -775,7 +775,7 @@
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="19" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -859,7 +859,7 @@
         <v>301125</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>306346.1538461539</v>
+        <v>306942.8571428572</v>
       </c>
     </row>
   </sheetData>
@@ -971,7 +971,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G438"/>
+  <dimension ref="A1:G447"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -16315,6 +16315,321 @@
         </is>
       </c>
     </row>
+    <row r="439">
+      <c r="A439" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B439" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C439" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D439" s="2" t="inlineStr">
+        <is>
+          <t>MT373</t>
+        </is>
+      </c>
+      <c r="E439" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F439" s="3" t="n">
+        <v>235500</v>
+      </c>
+      <c r="G439" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B440" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C440" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D440" s="2" t="inlineStr">
+        <is>
+          <t>MT374</t>
+        </is>
+      </c>
+      <c r="E440" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F440" s="3" t="n">
+        <v>259500</v>
+      </c>
+      <c r="G440" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B441" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C441" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D441" s="2" t="inlineStr">
+        <is>
+          <t>MT375</t>
+        </is>
+      </c>
+      <c r="E441" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F441" s="3" t="n">
+        <v>285500</v>
+      </c>
+      <c r="G441" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B442" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C442" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D442" s="2" t="inlineStr">
+        <is>
+          <t>MT376</t>
+        </is>
+      </c>
+      <c r="E442" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F442" s="3" t="n">
+        <v>339500</v>
+      </c>
+      <c r="G442" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B443" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C443" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D443" s="2" t="inlineStr">
+        <is>
+          <t>MTY69</t>
+        </is>
+      </c>
+      <c r="E443" s="2" t="inlineStr">
+        <is>
+          <t>Model Y L</t>
+        </is>
+      </c>
+      <c r="F443" s="3" t="n">
+        <v>339000</v>
+      </c>
+      <c r="G443" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B444" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C444" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D444" s="2" t="inlineStr">
+        <is>
+          <t>MTY79</t>
+        </is>
+      </c>
+      <c r="E444" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F444" s="3" t="n">
+        <v>263500</v>
+      </c>
+      <c r="G444" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B445" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C445" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D445" s="2" t="inlineStr">
+        <is>
+          <t>MTY80</t>
+        </is>
+      </c>
+      <c r="E445" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F445" s="3" t="n">
+        <v>313500</v>
+      </c>
+      <c r="G445" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B446" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C446" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D446" s="2" t="inlineStr">
+        <is>
+          <t>MTY81</t>
+        </is>
+      </c>
+      <c r="E446" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F446" s="3" t="n">
+        <v>288500</v>
+      </c>
+      <c r="G446" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B447" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C447" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D447" s="2" t="inlineStr">
+        <is>
+          <t>MTY88</t>
+        </is>
+      </c>
+      <c r="E447" s="2" t="inlineStr">
+        <is>
+          <t>Model Y Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F447" s="3" t="n">
+        <v>369000</v>
+      </c>
+      <c r="G447" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price pull 2026-09-17
</commit_message>
<xml_diff>
--- a/tesla_price_analysis.xlsx
+++ b/tesla_price_analysis.xlsx
@@ -445,7 +445,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Snapshot date: 2026-09-16  (source: tesla.com configurator pages)</t>
+          <t>Snapshot date: 2026-09-17  (source: tesla.com configurator pages)</t>
         </is>
       </c>
       <c r="B1" s="1" t="n"/>
@@ -775,7 +775,7 @@
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -859,7 +859,7 @@
         <v>301125</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>306942.8571428572</v>
+        <v>307460</v>
       </c>
     </row>
   </sheetData>
@@ -971,7 +971,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G447"/>
+  <dimension ref="A1:G456"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -16630,6 +16630,321 @@
         </is>
       </c>
     </row>
+    <row r="448">
+      <c r="A448" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B448" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C448" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D448" s="2" t="inlineStr">
+        <is>
+          <t>MT373</t>
+        </is>
+      </c>
+      <c r="E448" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F448" s="3" t="n">
+        <v>235500</v>
+      </c>
+      <c r="G448" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B449" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C449" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D449" s="2" t="inlineStr">
+        <is>
+          <t>MT374</t>
+        </is>
+      </c>
+      <c r="E449" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F449" s="3" t="n">
+        <v>259500</v>
+      </c>
+      <c r="G449" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B450" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C450" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D450" s="2" t="inlineStr">
+        <is>
+          <t>MT375</t>
+        </is>
+      </c>
+      <c r="E450" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F450" s="3" t="n">
+        <v>285500</v>
+      </c>
+      <c r="G450" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B451" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C451" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D451" s="2" t="inlineStr">
+        <is>
+          <t>MT376</t>
+        </is>
+      </c>
+      <c r="E451" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F451" s="3" t="n">
+        <v>339500</v>
+      </c>
+      <c r="G451" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B452" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C452" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D452" s="2" t="inlineStr">
+        <is>
+          <t>MTY69</t>
+        </is>
+      </c>
+      <c r="E452" s="2" t="inlineStr">
+        <is>
+          <t>Model Y L</t>
+        </is>
+      </c>
+      <c r="F452" s="3" t="n">
+        <v>339000</v>
+      </c>
+      <c r="G452" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B453" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C453" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D453" s="2" t="inlineStr">
+        <is>
+          <t>MTY79</t>
+        </is>
+      </c>
+      <c r="E453" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F453" s="3" t="n">
+        <v>263500</v>
+      </c>
+      <c r="G453" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B454" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C454" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D454" s="2" t="inlineStr">
+        <is>
+          <t>MTY80</t>
+        </is>
+      </c>
+      <c r="E454" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F454" s="3" t="n">
+        <v>313500</v>
+      </c>
+      <c r="G454" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B455" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C455" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D455" s="2" t="inlineStr">
+        <is>
+          <t>MTY81</t>
+        </is>
+      </c>
+      <c r="E455" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F455" s="3" t="n">
+        <v>288500</v>
+      </c>
+      <c r="G455" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B456" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C456" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D456" s="2" t="inlineStr">
+        <is>
+          <t>MTY88</t>
+        </is>
+      </c>
+      <c r="E456" s="2" t="inlineStr">
+        <is>
+          <t>Model Y Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F456" s="3" t="n">
+        <v>369000</v>
+      </c>
+      <c r="G456" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price pull 2026-09-18
</commit_message>
<xml_diff>
--- a/tesla_price_analysis.xlsx
+++ b/tesla_price_analysis.xlsx
@@ -445,7 +445,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Snapshot date: 2026-09-17  (source: tesla.com configurator pages)</t>
+          <t>Snapshot date: 2026-09-18  (source: tesla.com configurator pages)</t>
         </is>
       </c>
       <c r="B1" s="1" t="n"/>
@@ -859,7 +859,7 @@
         <v>301125</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>307460</v>
+        <v>307912.5</v>
       </c>
     </row>
   </sheetData>
@@ -971,7 +971,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G456"/>
+  <dimension ref="A1:G465"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -16945,6 +16945,321 @@
         </is>
       </c>
     </row>
+    <row r="457">
+      <c r="A457" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B457" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C457" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D457" s="2" t="inlineStr">
+        <is>
+          <t>MT373</t>
+        </is>
+      </c>
+      <c r="E457" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F457" s="3" t="n">
+        <v>235500</v>
+      </c>
+      <c r="G457" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B458" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C458" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D458" s="2" t="inlineStr">
+        <is>
+          <t>MT374</t>
+        </is>
+      </c>
+      <c r="E458" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F458" s="3" t="n">
+        <v>259500</v>
+      </c>
+      <c r="G458" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B459" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C459" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D459" s="2" t="inlineStr">
+        <is>
+          <t>MT375</t>
+        </is>
+      </c>
+      <c r="E459" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F459" s="3" t="n">
+        <v>285500</v>
+      </c>
+      <c r="G459" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B460" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C460" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D460" s="2" t="inlineStr">
+        <is>
+          <t>MT376</t>
+        </is>
+      </c>
+      <c r="E460" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F460" s="3" t="n">
+        <v>339500</v>
+      </c>
+      <c r="G460" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B461" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C461" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D461" s="2" t="inlineStr">
+        <is>
+          <t>MTY69</t>
+        </is>
+      </c>
+      <c r="E461" s="2" t="inlineStr">
+        <is>
+          <t>Model Y L</t>
+        </is>
+      </c>
+      <c r="F461" s="3" t="n">
+        <v>339000</v>
+      </c>
+      <c r="G461" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B462" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C462" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D462" s="2" t="inlineStr">
+        <is>
+          <t>MTY79</t>
+        </is>
+      </c>
+      <c r="E462" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F462" s="3" t="n">
+        <v>263500</v>
+      </c>
+      <c r="G462" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B463" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C463" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D463" s="2" t="inlineStr">
+        <is>
+          <t>MTY80</t>
+        </is>
+      </c>
+      <c r="E463" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F463" s="3" t="n">
+        <v>313500</v>
+      </c>
+      <c r="G463" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B464" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C464" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D464" s="2" t="inlineStr">
+        <is>
+          <t>MTY81</t>
+        </is>
+      </c>
+      <c r="E464" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F464" s="3" t="n">
+        <v>288500</v>
+      </c>
+      <c r="G464" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B465" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C465" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D465" s="2" t="inlineStr">
+        <is>
+          <t>MTY88</t>
+        </is>
+      </c>
+      <c r="E465" s="2" t="inlineStr">
+        <is>
+          <t>Model Y Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F465" s="3" t="n">
+        <v>369000</v>
+      </c>
+      <c r="G465" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price pull 2026-09-19
</commit_message>
<xml_diff>
--- a/tesla_price_analysis.xlsx
+++ b/tesla_price_analysis.xlsx
@@ -445,7 +445,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Snapshot date: 2026-09-18  (source: tesla.com configurator pages)</t>
+          <t>Snapshot date: 2026-09-19  (source: tesla.com configurator pages)</t>
         </is>
       </c>
       <c r="B1" s="1" t="n"/>
@@ -775,7 +775,7 @@
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -859,7 +859,7 @@
         <v>301125</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>307912.5</v>
+        <v>308311.7647058823</v>
       </c>
     </row>
   </sheetData>
@@ -971,7 +971,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G465"/>
+  <dimension ref="A1:G474"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -17260,6 +17260,321 @@
         </is>
       </c>
     </row>
+    <row r="466">
+      <c r="A466" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B466" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C466" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D466" s="2" t="inlineStr">
+        <is>
+          <t>MT373</t>
+        </is>
+      </c>
+      <c r="E466" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F466" s="3" t="n">
+        <v>235500</v>
+      </c>
+      <c r="G466" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B467" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C467" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D467" s="2" t="inlineStr">
+        <is>
+          <t>MT374</t>
+        </is>
+      </c>
+      <c r="E467" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F467" s="3" t="n">
+        <v>259500</v>
+      </c>
+      <c r="G467" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B468" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C468" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D468" s="2" t="inlineStr">
+        <is>
+          <t>MT375</t>
+        </is>
+      </c>
+      <c r="E468" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F468" s="3" t="n">
+        <v>285500</v>
+      </c>
+      <c r="G468" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B469" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C469" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D469" s="2" t="inlineStr">
+        <is>
+          <t>MT376</t>
+        </is>
+      </c>
+      <c r="E469" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F469" s="3" t="n">
+        <v>339500</v>
+      </c>
+      <c r="G469" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B470" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C470" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D470" s="2" t="inlineStr">
+        <is>
+          <t>MTY69</t>
+        </is>
+      </c>
+      <c r="E470" s="2" t="inlineStr">
+        <is>
+          <t>Model Y L</t>
+        </is>
+      </c>
+      <c r="F470" s="3" t="n">
+        <v>339000</v>
+      </c>
+      <c r="G470" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B471" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C471" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D471" s="2" t="inlineStr">
+        <is>
+          <t>MTY79</t>
+        </is>
+      </c>
+      <c r="E471" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F471" s="3" t="n">
+        <v>263500</v>
+      </c>
+      <c r="G471" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B472" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C472" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D472" s="2" t="inlineStr">
+        <is>
+          <t>MTY80</t>
+        </is>
+      </c>
+      <c r="E472" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F472" s="3" t="n">
+        <v>313500</v>
+      </c>
+      <c r="G472" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B473" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C473" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D473" s="2" t="inlineStr">
+        <is>
+          <t>MTY81</t>
+        </is>
+      </c>
+      <c r="E473" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F473" s="3" t="n">
+        <v>288500</v>
+      </c>
+      <c r="G473" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B474" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C474" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D474" s="2" t="inlineStr">
+        <is>
+          <t>MTY88</t>
+        </is>
+      </c>
+      <c r="E474" s="2" t="inlineStr">
+        <is>
+          <t>Model Y Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F474" s="3" t="n">
+        <v>369000</v>
+      </c>
+      <c r="G474" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price pull 2026-09-20
</commit_message>
<xml_diff>
--- a/tesla_price_analysis.xlsx
+++ b/tesla_price_analysis.xlsx
@@ -445,7 +445,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Snapshot date: 2026-09-19  (source: tesla.com configurator pages)</t>
+          <t>Snapshot date: 2026-09-20  (source: tesla.com configurator pages)</t>
         </is>
       </c>
       <c r="B1" s="1" t="n"/>
@@ -775,7 +775,7 @@
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="19" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -859,7 +859,7 @@
         <v>301125</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>308311.7647058823</v>
+        <v>308666.6666666667</v>
       </c>
     </row>
   </sheetData>
@@ -971,7 +971,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G474"/>
+  <dimension ref="A1:G483"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -17575,6 +17575,321 @@
         </is>
       </c>
     </row>
+    <row r="475">
+      <c r="A475" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B475" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C475" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D475" s="2" t="inlineStr">
+        <is>
+          <t>MT373</t>
+        </is>
+      </c>
+      <c r="E475" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F475" s="3" t="n">
+        <v>235500</v>
+      </c>
+      <c r="G475" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B476" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C476" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D476" s="2" t="inlineStr">
+        <is>
+          <t>MT374</t>
+        </is>
+      </c>
+      <c r="E476" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F476" s="3" t="n">
+        <v>259500</v>
+      </c>
+      <c r="G476" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B477" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C477" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D477" s="2" t="inlineStr">
+        <is>
+          <t>MT375</t>
+        </is>
+      </c>
+      <c r="E477" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F477" s="3" t="n">
+        <v>285500</v>
+      </c>
+      <c r="G477" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B478" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C478" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D478" s="2" t="inlineStr">
+        <is>
+          <t>MT376</t>
+        </is>
+      </c>
+      <c r="E478" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F478" s="3" t="n">
+        <v>339500</v>
+      </c>
+      <c r="G478" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B479" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C479" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D479" s="2" t="inlineStr">
+        <is>
+          <t>MTY69</t>
+        </is>
+      </c>
+      <c r="E479" s="2" t="inlineStr">
+        <is>
+          <t>Model Y L</t>
+        </is>
+      </c>
+      <c r="F479" s="3" t="n">
+        <v>339000</v>
+      </c>
+      <c r="G479" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B480" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C480" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D480" s="2" t="inlineStr">
+        <is>
+          <t>MTY79</t>
+        </is>
+      </c>
+      <c r="E480" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F480" s="3" t="n">
+        <v>263500</v>
+      </c>
+      <c r="G480" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B481" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C481" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D481" s="2" t="inlineStr">
+        <is>
+          <t>MTY80</t>
+        </is>
+      </c>
+      <c r="E481" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F481" s="3" t="n">
+        <v>313500</v>
+      </c>
+      <c r="G481" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B482" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C482" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D482" s="2" t="inlineStr">
+        <is>
+          <t>MTY81</t>
+        </is>
+      </c>
+      <c r="E482" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F482" s="3" t="n">
+        <v>288500</v>
+      </c>
+      <c r="G482" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B483" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C483" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D483" s="2" t="inlineStr">
+        <is>
+          <t>MTY88</t>
+        </is>
+      </c>
+      <c r="E483" s="2" t="inlineStr">
+        <is>
+          <t>Model Y Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F483" s="3" t="n">
+        <v>369000</v>
+      </c>
+      <c r="G483" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price pull 2026-09-21
</commit_message>
<xml_diff>
--- a/tesla_price_analysis.xlsx
+++ b/tesla_price_analysis.xlsx
@@ -445,7 +445,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Snapshot date: 2026-09-20  (source: tesla.com configurator pages)</t>
+          <t>Snapshot date: 2026-09-21  (source: tesla.com configurator pages)</t>
         </is>
       </c>
       <c r="B1" s="1" t="n"/>
@@ -859,7 +859,7 @@
         <v>301125</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>308666.6666666667</v>
+        <v>308984.2105263158</v>
       </c>
     </row>
   </sheetData>
@@ -971,7 +971,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G483"/>
+  <dimension ref="A1:G492"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -17890,6 +17890,321 @@
         </is>
       </c>
     </row>
+    <row r="484">
+      <c r="A484" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B484" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C484" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D484" s="2" t="inlineStr">
+        <is>
+          <t>MT373</t>
+        </is>
+      </c>
+      <c r="E484" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F484" s="3" t="n">
+        <v>235500</v>
+      </c>
+      <c r="G484" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B485" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C485" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D485" s="2" t="inlineStr">
+        <is>
+          <t>MT374</t>
+        </is>
+      </c>
+      <c r="E485" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F485" s="3" t="n">
+        <v>259500</v>
+      </c>
+      <c r="G485" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B486" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C486" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D486" s="2" t="inlineStr">
+        <is>
+          <t>MT375</t>
+        </is>
+      </c>
+      <c r="E486" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F486" s="3" t="n">
+        <v>285500</v>
+      </c>
+      <c r="G486" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B487" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C487" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D487" s="2" t="inlineStr">
+        <is>
+          <t>MT376</t>
+        </is>
+      </c>
+      <c r="E487" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F487" s="3" t="n">
+        <v>339500</v>
+      </c>
+      <c r="G487" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B488" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C488" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D488" s="2" t="inlineStr">
+        <is>
+          <t>MTY69</t>
+        </is>
+      </c>
+      <c r="E488" s="2" t="inlineStr">
+        <is>
+          <t>Model Y L</t>
+        </is>
+      </c>
+      <c r="F488" s="3" t="n">
+        <v>339000</v>
+      </c>
+      <c r="G488" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B489" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C489" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D489" s="2" t="inlineStr">
+        <is>
+          <t>MTY79</t>
+        </is>
+      </c>
+      <c r="E489" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F489" s="3" t="n">
+        <v>263500</v>
+      </c>
+      <c r="G489" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B490" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C490" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D490" s="2" t="inlineStr">
+        <is>
+          <t>MTY80</t>
+        </is>
+      </c>
+      <c r="E490" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F490" s="3" t="n">
+        <v>313500</v>
+      </c>
+      <c r="G490" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B491" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C491" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D491" s="2" t="inlineStr">
+        <is>
+          <t>MTY81</t>
+        </is>
+      </c>
+      <c r="E491" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F491" s="3" t="n">
+        <v>288500</v>
+      </c>
+      <c r="G491" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B492" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C492" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D492" s="2" t="inlineStr">
+        <is>
+          <t>MTY88</t>
+        </is>
+      </c>
+      <c r="E492" s="2" t="inlineStr">
+        <is>
+          <t>Model Y Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F492" s="3" t="n">
+        <v>369000</v>
+      </c>
+      <c r="G492" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price pull 2026-09-22
</commit_message>
<xml_diff>
--- a/tesla_price_analysis.xlsx
+++ b/tesla_price_analysis.xlsx
@@ -445,7 +445,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Snapshot date: 2026-09-21  (source: tesla.com configurator pages)</t>
+          <t>Snapshot date: 2026-09-22  (source: tesla.com configurator pages)</t>
         </is>
       </c>
       <c r="B1" s="1" t="n"/>
@@ -775,7 +775,7 @@
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="19" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -859,7 +859,7 @@
         <v>301125</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>308984.2105263158</v>
+        <v>309270</v>
       </c>
     </row>
   </sheetData>
@@ -971,7 +971,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G492"/>
+  <dimension ref="A1:G501"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -18205,6 +18205,321 @@
         </is>
       </c>
     </row>
+    <row r="493">
+      <c r="A493" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B493" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C493" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D493" s="2" t="inlineStr">
+        <is>
+          <t>MT373</t>
+        </is>
+      </c>
+      <c r="E493" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F493" s="3" t="n">
+        <v>235500</v>
+      </c>
+      <c r="G493" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B494" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C494" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D494" s="2" t="inlineStr">
+        <is>
+          <t>MT374</t>
+        </is>
+      </c>
+      <c r="E494" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F494" s="3" t="n">
+        <v>259500</v>
+      </c>
+      <c r="G494" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B495" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C495" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D495" s="2" t="inlineStr">
+        <is>
+          <t>MT375</t>
+        </is>
+      </c>
+      <c r="E495" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F495" s="3" t="n">
+        <v>285500</v>
+      </c>
+      <c r="G495" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B496" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C496" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D496" s="2" t="inlineStr">
+        <is>
+          <t>MT376</t>
+        </is>
+      </c>
+      <c r="E496" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F496" s="3" t="n">
+        <v>339500</v>
+      </c>
+      <c r="G496" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B497" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C497" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D497" s="2" t="inlineStr">
+        <is>
+          <t>MTY69</t>
+        </is>
+      </c>
+      <c r="E497" s="2" t="inlineStr">
+        <is>
+          <t>Model Y L</t>
+        </is>
+      </c>
+      <c r="F497" s="3" t="n">
+        <v>339000</v>
+      </c>
+      <c r="G497" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B498" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C498" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D498" s="2" t="inlineStr">
+        <is>
+          <t>MTY79</t>
+        </is>
+      </c>
+      <c r="E498" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F498" s="3" t="n">
+        <v>263500</v>
+      </c>
+      <c r="G498" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B499" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C499" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D499" s="2" t="inlineStr">
+        <is>
+          <t>MTY80</t>
+        </is>
+      </c>
+      <c r="E499" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F499" s="3" t="n">
+        <v>313500</v>
+      </c>
+      <c r="G499" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B500" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C500" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D500" s="2" t="inlineStr">
+        <is>
+          <t>MTY81</t>
+        </is>
+      </c>
+      <c r="E500" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F500" s="3" t="n">
+        <v>288500</v>
+      </c>
+      <c r="G500" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B501" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C501" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D501" s="2" t="inlineStr">
+        <is>
+          <t>MTY88</t>
+        </is>
+      </c>
+      <c r="E501" s="2" t="inlineStr">
+        <is>
+          <t>Model Y Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F501" s="3" t="n">
+        <v>369000</v>
+      </c>
+      <c r="G501" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price pull 2026-09-23
</commit_message>
<xml_diff>
--- a/tesla_price_analysis.xlsx
+++ b/tesla_price_analysis.xlsx
@@ -445,7 +445,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Snapshot date: 2026-09-22  (source: tesla.com configurator pages)</t>
+          <t>Snapshot date: 2026-09-23  (source: tesla.com configurator pages)</t>
         </is>
       </c>
       <c r="B1" s="1" t="n"/>
@@ -775,7 +775,7 @@
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="19" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -859,7 +859,7 @@
         <v>301125</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>309270</v>
+        <v>309528.5714285714</v>
       </c>
     </row>
   </sheetData>
@@ -971,7 +971,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G501"/>
+  <dimension ref="A1:G510"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -18520,6 +18520,321 @@
         </is>
       </c>
     </row>
+    <row r="502">
+      <c r="A502" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B502" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C502" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D502" s="2" t="inlineStr">
+        <is>
+          <t>MT373</t>
+        </is>
+      </c>
+      <c r="E502" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F502" s="3" t="n">
+        <v>235500</v>
+      </c>
+      <c r="G502" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B503" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C503" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D503" s="2" t="inlineStr">
+        <is>
+          <t>MT374</t>
+        </is>
+      </c>
+      <c r="E503" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F503" s="3" t="n">
+        <v>259500</v>
+      </c>
+      <c r="G503" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B504" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C504" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D504" s="2" t="inlineStr">
+        <is>
+          <t>MT375</t>
+        </is>
+      </c>
+      <c r="E504" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F504" s="3" t="n">
+        <v>285500</v>
+      </c>
+      <c r="G504" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B505" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C505" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D505" s="2" t="inlineStr">
+        <is>
+          <t>MT376</t>
+        </is>
+      </c>
+      <c r="E505" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F505" s="3" t="n">
+        <v>339500</v>
+      </c>
+      <c r="G505" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B506" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C506" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D506" s="2" t="inlineStr">
+        <is>
+          <t>MTY69</t>
+        </is>
+      </c>
+      <c r="E506" s="2" t="inlineStr">
+        <is>
+          <t>Model Y L</t>
+        </is>
+      </c>
+      <c r="F506" s="3" t="n">
+        <v>339000</v>
+      </c>
+      <c r="G506" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B507" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C507" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D507" s="2" t="inlineStr">
+        <is>
+          <t>MTY79</t>
+        </is>
+      </c>
+      <c r="E507" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F507" s="3" t="n">
+        <v>263500</v>
+      </c>
+      <c r="G507" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B508" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C508" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D508" s="2" t="inlineStr">
+        <is>
+          <t>MTY80</t>
+        </is>
+      </c>
+      <c r="E508" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F508" s="3" t="n">
+        <v>313500</v>
+      </c>
+      <c r="G508" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B509" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C509" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D509" s="2" t="inlineStr">
+        <is>
+          <t>MTY81</t>
+        </is>
+      </c>
+      <c r="E509" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F509" s="3" t="n">
+        <v>288500</v>
+      </c>
+      <c r="G509" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B510" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C510" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D510" s="2" t="inlineStr">
+        <is>
+          <t>MTY88</t>
+        </is>
+      </c>
+      <c r="E510" s="2" t="inlineStr">
+        <is>
+          <t>Model Y Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F510" s="3" t="n">
+        <v>369000</v>
+      </c>
+      <c r="G510" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price pull 2026-09-24
</commit_message>
<xml_diff>
--- a/tesla_price_analysis.xlsx
+++ b/tesla_price_analysis.xlsx
@@ -445,7 +445,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Snapshot date: 2026-09-23  (source: tesla.com configurator pages)</t>
+          <t>Snapshot date: 2026-09-24  (source: tesla.com configurator pages)</t>
         </is>
       </c>
       <c r="B1" s="1" t="n"/>
@@ -775,7 +775,7 @@
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="19" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -859,7 +859,7 @@
         <v>301125</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>309528.5714285714</v>
+        <v>309763.6363636364</v>
       </c>
     </row>
   </sheetData>
@@ -971,7 +971,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G510"/>
+  <dimension ref="A1:G519"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -18835,6 +18835,321 @@
         </is>
       </c>
     </row>
+    <row r="511">
+      <c r="A511" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B511" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C511" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D511" s="2" t="inlineStr">
+        <is>
+          <t>MT373</t>
+        </is>
+      </c>
+      <c r="E511" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F511" s="3" t="n">
+        <v>235500</v>
+      </c>
+      <c r="G511" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B512" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C512" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D512" s="2" t="inlineStr">
+        <is>
+          <t>MT374</t>
+        </is>
+      </c>
+      <c r="E512" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F512" s="3" t="n">
+        <v>259500</v>
+      </c>
+      <c r="G512" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B513" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C513" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D513" s="2" t="inlineStr">
+        <is>
+          <t>MT375</t>
+        </is>
+      </c>
+      <c r="E513" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F513" s="3" t="n">
+        <v>285500</v>
+      </c>
+      <c r="G513" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B514" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C514" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D514" s="2" t="inlineStr">
+        <is>
+          <t>MT376</t>
+        </is>
+      </c>
+      <c r="E514" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F514" s="3" t="n">
+        <v>339500</v>
+      </c>
+      <c r="G514" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B515" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C515" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D515" s="2" t="inlineStr">
+        <is>
+          <t>MTY69</t>
+        </is>
+      </c>
+      <c r="E515" s="2" t="inlineStr">
+        <is>
+          <t>Model Y L</t>
+        </is>
+      </c>
+      <c r="F515" s="3" t="n">
+        <v>339000</v>
+      </c>
+      <c r="G515" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B516" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C516" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D516" s="2" t="inlineStr">
+        <is>
+          <t>MTY79</t>
+        </is>
+      </c>
+      <c r="E516" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F516" s="3" t="n">
+        <v>263500</v>
+      </c>
+      <c r="G516" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B517" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C517" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D517" s="2" t="inlineStr">
+        <is>
+          <t>MTY80</t>
+        </is>
+      </c>
+      <c r="E517" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F517" s="3" t="n">
+        <v>313500</v>
+      </c>
+      <c r="G517" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B518" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C518" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D518" s="2" t="inlineStr">
+        <is>
+          <t>MTY81</t>
+        </is>
+      </c>
+      <c r="E518" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F518" s="3" t="n">
+        <v>288500</v>
+      </c>
+      <c r="G518" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B519" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C519" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D519" s="2" t="inlineStr">
+        <is>
+          <t>MTY88</t>
+        </is>
+      </c>
+      <c r="E519" s="2" t="inlineStr">
+        <is>
+          <t>Model Y Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F519" s="3" t="n">
+        <v>369000</v>
+      </c>
+      <c r="G519" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price pull 2026-09-25
</commit_message>
<xml_diff>
--- a/tesla_price_analysis.xlsx
+++ b/tesla_price_analysis.xlsx
@@ -445,7 +445,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Snapshot date: 2026-09-24  (source: tesla.com configurator pages)</t>
+          <t>Snapshot date: 2026-09-25  (source: tesla.com configurator pages)</t>
         </is>
       </c>
       <c r="B1" s="1" t="n"/>
@@ -859,7 +859,7 @@
         <v>301125</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>309763.6363636364</v>
+        <v>309978.2608695652</v>
       </c>
     </row>
   </sheetData>
@@ -971,7 +971,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G519"/>
+  <dimension ref="A1:G528"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -19150,6 +19150,321 @@
         </is>
       </c>
     </row>
+    <row r="520">
+      <c r="A520" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B520" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C520" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D520" s="2" t="inlineStr">
+        <is>
+          <t>MT373</t>
+        </is>
+      </c>
+      <c r="E520" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F520" s="3" t="n">
+        <v>235500</v>
+      </c>
+      <c r="G520" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="521">
+      <c r="A521" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B521" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C521" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D521" s="2" t="inlineStr">
+        <is>
+          <t>MT374</t>
+        </is>
+      </c>
+      <c r="E521" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F521" s="3" t="n">
+        <v>259500</v>
+      </c>
+      <c r="G521" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B522" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C522" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D522" s="2" t="inlineStr">
+        <is>
+          <t>MT375</t>
+        </is>
+      </c>
+      <c r="E522" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F522" s="3" t="n">
+        <v>285500</v>
+      </c>
+      <c r="G522" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B523" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C523" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D523" s="2" t="inlineStr">
+        <is>
+          <t>MT376</t>
+        </is>
+      </c>
+      <c r="E523" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F523" s="3" t="n">
+        <v>339500</v>
+      </c>
+      <c r="G523" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B524" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C524" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D524" s="2" t="inlineStr">
+        <is>
+          <t>MTY69</t>
+        </is>
+      </c>
+      <c r="E524" s="2" t="inlineStr">
+        <is>
+          <t>Model Y L</t>
+        </is>
+      </c>
+      <c r="F524" s="3" t="n">
+        <v>339000</v>
+      </c>
+      <c r="G524" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="525">
+      <c r="A525" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B525" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C525" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D525" s="2" t="inlineStr">
+        <is>
+          <t>MTY79</t>
+        </is>
+      </c>
+      <c r="E525" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F525" s="3" t="n">
+        <v>263500</v>
+      </c>
+      <c r="G525" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="526">
+      <c r="A526" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B526" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C526" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D526" s="2" t="inlineStr">
+        <is>
+          <t>MTY80</t>
+        </is>
+      </c>
+      <c r="E526" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F526" s="3" t="n">
+        <v>313500</v>
+      </c>
+      <c r="G526" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="527">
+      <c r="A527" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B527" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C527" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D527" s="2" t="inlineStr">
+        <is>
+          <t>MTY81</t>
+        </is>
+      </c>
+      <c r="E527" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F527" s="3" t="n">
+        <v>288500</v>
+      </c>
+      <c r="G527" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="528">
+      <c r="A528" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B528" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C528" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D528" s="2" t="inlineStr">
+        <is>
+          <t>MTY88</t>
+        </is>
+      </c>
+      <c r="E528" s="2" t="inlineStr">
+        <is>
+          <t>Model Y Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F528" s="3" t="n">
+        <v>369000</v>
+      </c>
+      <c r="G528" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price pull 2026-09-26
</commit_message>
<xml_diff>
--- a/tesla_price_analysis.xlsx
+++ b/tesla_price_analysis.xlsx
@@ -445,7 +445,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Snapshot date: 2026-09-25  (source: tesla.com configurator pages)</t>
+          <t>Snapshot date: 2026-09-26  (source: tesla.com configurator pages)</t>
         </is>
       </c>
       <c r="B1" s="1" t="n"/>
@@ -775,7 +775,7 @@
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -859,7 +859,7 @@
         <v>301125</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>309978.2608695652</v>
+        <v>310175</v>
       </c>
     </row>
   </sheetData>
@@ -971,7 +971,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G528"/>
+  <dimension ref="A1:G537"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -19465,6 +19465,321 @@
         </is>
       </c>
     </row>
+    <row r="529">
+      <c r="A529" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B529" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C529" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D529" s="2" t="inlineStr">
+        <is>
+          <t>MT373</t>
+        </is>
+      </c>
+      <c r="E529" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F529" s="3" t="n">
+        <v>235500</v>
+      </c>
+      <c r="G529" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="530">
+      <c r="A530" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B530" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C530" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D530" s="2" t="inlineStr">
+        <is>
+          <t>MT374</t>
+        </is>
+      </c>
+      <c r="E530" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F530" s="3" t="n">
+        <v>259500</v>
+      </c>
+      <c r="G530" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="531">
+      <c r="A531" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B531" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C531" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D531" s="2" t="inlineStr">
+        <is>
+          <t>MT375</t>
+        </is>
+      </c>
+      <c r="E531" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F531" s="3" t="n">
+        <v>285500</v>
+      </c>
+      <c r="G531" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="532">
+      <c r="A532" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B532" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C532" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D532" s="2" t="inlineStr">
+        <is>
+          <t>MT376</t>
+        </is>
+      </c>
+      <c r="E532" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F532" s="3" t="n">
+        <v>339500</v>
+      </c>
+      <c r="G532" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="533">
+      <c r="A533" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B533" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C533" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D533" s="2" t="inlineStr">
+        <is>
+          <t>MTY69</t>
+        </is>
+      </c>
+      <c r="E533" s="2" t="inlineStr">
+        <is>
+          <t>Model Y L</t>
+        </is>
+      </c>
+      <c r="F533" s="3" t="n">
+        <v>339000</v>
+      </c>
+      <c r="G533" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="534">
+      <c r="A534" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B534" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C534" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D534" s="2" t="inlineStr">
+        <is>
+          <t>MTY79</t>
+        </is>
+      </c>
+      <c r="E534" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F534" s="3" t="n">
+        <v>263500</v>
+      </c>
+      <c r="G534" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="535">
+      <c r="A535" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B535" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C535" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D535" s="2" t="inlineStr">
+        <is>
+          <t>MTY80</t>
+        </is>
+      </c>
+      <c r="E535" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F535" s="3" t="n">
+        <v>313500</v>
+      </c>
+      <c r="G535" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="536">
+      <c r="A536" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B536" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C536" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D536" s="2" t="inlineStr">
+        <is>
+          <t>MTY81</t>
+        </is>
+      </c>
+      <c r="E536" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F536" s="3" t="n">
+        <v>288500</v>
+      </c>
+      <c r="G536" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="537">
+      <c r="A537" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B537" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C537" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D537" s="2" t="inlineStr">
+        <is>
+          <t>MTY88</t>
+        </is>
+      </c>
+      <c r="E537" s="2" t="inlineStr">
+        <is>
+          <t>Model Y Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F537" s="3" t="n">
+        <v>369000</v>
+      </c>
+      <c r="G537" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price pull 2026-09-27
</commit_message>
<xml_diff>
--- a/tesla_price_analysis.xlsx
+++ b/tesla_price_analysis.xlsx
@@ -445,7 +445,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Snapshot date: 2026-09-26  (source: tesla.com configurator pages)</t>
+          <t>Snapshot date: 2026-09-27  (source: tesla.com configurator pages)</t>
         </is>
       </c>
       <c r="B1" s="1" t="n"/>
@@ -859,7 +859,7 @@
         <v>301125</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>310175</v>
+        <v>310356</v>
       </c>
     </row>
   </sheetData>
@@ -971,7 +971,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G537"/>
+  <dimension ref="A1:G546"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -19780,6 +19780,321 @@
         </is>
       </c>
     </row>
+    <row r="538">
+      <c r="A538" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B538" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C538" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D538" s="2" t="inlineStr">
+        <is>
+          <t>MT373</t>
+        </is>
+      </c>
+      <c r="E538" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F538" s="3" t="n">
+        <v>235500</v>
+      </c>
+      <c r="G538" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="539">
+      <c r="A539" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B539" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C539" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D539" s="2" t="inlineStr">
+        <is>
+          <t>MT374</t>
+        </is>
+      </c>
+      <c r="E539" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F539" s="3" t="n">
+        <v>259500</v>
+      </c>
+      <c r="G539" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="540">
+      <c r="A540" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B540" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C540" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D540" s="2" t="inlineStr">
+        <is>
+          <t>MT375</t>
+        </is>
+      </c>
+      <c r="E540" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F540" s="3" t="n">
+        <v>285500</v>
+      </c>
+      <c r="G540" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="541">
+      <c r="A541" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B541" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C541" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D541" s="2" t="inlineStr">
+        <is>
+          <t>MT376</t>
+        </is>
+      </c>
+      <c r="E541" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F541" s="3" t="n">
+        <v>339500</v>
+      </c>
+      <c r="G541" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="542">
+      <c r="A542" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B542" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C542" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D542" s="2" t="inlineStr">
+        <is>
+          <t>MTY69</t>
+        </is>
+      </c>
+      <c r="E542" s="2" t="inlineStr">
+        <is>
+          <t>Model Y L</t>
+        </is>
+      </c>
+      <c r="F542" s="3" t="n">
+        <v>339000</v>
+      </c>
+      <c r="G542" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="543">
+      <c r="A543" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B543" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C543" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D543" s="2" t="inlineStr">
+        <is>
+          <t>MTY79</t>
+        </is>
+      </c>
+      <c r="E543" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F543" s="3" t="n">
+        <v>263500</v>
+      </c>
+      <c r="G543" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="544">
+      <c r="A544" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B544" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C544" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D544" s="2" t="inlineStr">
+        <is>
+          <t>MTY80</t>
+        </is>
+      </c>
+      <c r="E544" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F544" s="3" t="n">
+        <v>313500</v>
+      </c>
+      <c r="G544" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="545">
+      <c r="A545" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B545" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C545" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D545" s="2" t="inlineStr">
+        <is>
+          <t>MTY81</t>
+        </is>
+      </c>
+      <c r="E545" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F545" s="3" t="n">
+        <v>288500</v>
+      </c>
+      <c r="G545" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="546">
+      <c r="A546" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B546" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C546" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D546" s="2" t="inlineStr">
+        <is>
+          <t>MTY88</t>
+        </is>
+      </c>
+      <c r="E546" s="2" t="inlineStr">
+        <is>
+          <t>Model Y Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F546" s="3" t="n">
+        <v>369000</v>
+      </c>
+      <c r="G546" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price pull 2026-09-28
</commit_message>
<xml_diff>
--- a/tesla_price_analysis.xlsx
+++ b/tesla_price_analysis.xlsx
@@ -445,7 +445,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Snapshot date: 2026-09-27  (source: tesla.com configurator pages)</t>
+          <t>Snapshot date: 2026-09-28  (source: tesla.com configurator pages)</t>
         </is>
       </c>
       <c r="B1" s="1" t="n"/>
@@ -775,7 +775,7 @@
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -859,7 +859,7 @@
         <v>301125</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>310356</v>
+        <v>310523.0769230769</v>
       </c>
     </row>
   </sheetData>
@@ -971,7 +971,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G546"/>
+  <dimension ref="A1:G555"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -20095,6 +20095,321 @@
         </is>
       </c>
     </row>
+    <row r="547">
+      <c r="A547" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B547" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C547" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D547" s="2" t="inlineStr">
+        <is>
+          <t>MT373</t>
+        </is>
+      </c>
+      <c r="E547" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F547" s="3" t="n">
+        <v>235500</v>
+      </c>
+      <c r="G547" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="548">
+      <c r="A548" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B548" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C548" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D548" s="2" t="inlineStr">
+        <is>
+          <t>MT374</t>
+        </is>
+      </c>
+      <c r="E548" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F548" s="3" t="n">
+        <v>259500</v>
+      </c>
+      <c r="G548" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B549" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C549" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D549" s="2" t="inlineStr">
+        <is>
+          <t>MT375</t>
+        </is>
+      </c>
+      <c r="E549" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F549" s="3" t="n">
+        <v>285500</v>
+      </c>
+      <c r="G549" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="550">
+      <c r="A550" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B550" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C550" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D550" s="2" t="inlineStr">
+        <is>
+          <t>MT376</t>
+        </is>
+      </c>
+      <c r="E550" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F550" s="3" t="n">
+        <v>339500</v>
+      </c>
+      <c r="G550" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="551">
+      <c r="A551" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B551" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C551" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D551" s="2" t="inlineStr">
+        <is>
+          <t>MTY69</t>
+        </is>
+      </c>
+      <c r="E551" s="2" t="inlineStr">
+        <is>
+          <t>Model Y L</t>
+        </is>
+      </c>
+      <c r="F551" s="3" t="n">
+        <v>339000</v>
+      </c>
+      <c r="G551" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="552">
+      <c r="A552" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B552" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C552" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D552" s="2" t="inlineStr">
+        <is>
+          <t>MTY79</t>
+        </is>
+      </c>
+      <c r="E552" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F552" s="3" t="n">
+        <v>263500</v>
+      </c>
+      <c r="G552" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="553">
+      <c r="A553" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B553" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C553" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D553" s="2" t="inlineStr">
+        <is>
+          <t>MTY80</t>
+        </is>
+      </c>
+      <c r="E553" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F553" s="3" t="n">
+        <v>313500</v>
+      </c>
+      <c r="G553" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="554">
+      <c r="A554" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B554" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C554" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D554" s="2" t="inlineStr">
+        <is>
+          <t>MTY81</t>
+        </is>
+      </c>
+      <c r="E554" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F554" s="3" t="n">
+        <v>288500</v>
+      </c>
+      <c r="G554" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="555">
+      <c r="A555" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B555" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C555" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D555" s="2" t="inlineStr">
+        <is>
+          <t>MTY88</t>
+        </is>
+      </c>
+      <c r="E555" s="2" t="inlineStr">
+        <is>
+          <t>Model Y Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F555" s="3" t="n">
+        <v>369000</v>
+      </c>
+      <c r="G555" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price pull 2026-09-29
</commit_message>
<xml_diff>
--- a/tesla_price_analysis.xlsx
+++ b/tesla_price_analysis.xlsx
@@ -445,7 +445,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Snapshot date: 2026-09-28  (source: tesla.com configurator pages)</t>
+          <t>Snapshot date: 2026-09-29  (source: tesla.com configurator pages)</t>
         </is>
       </c>
       <c r="B1" s="1" t="n"/>
@@ -859,7 +859,7 @@
         <v>301125</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>310523.0769230769</v>
+        <v>310677.7777777778</v>
       </c>
     </row>
   </sheetData>
@@ -971,7 +971,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G555"/>
+  <dimension ref="A1:G564"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -20410,6 +20410,321 @@
         </is>
       </c>
     </row>
+    <row r="556">
+      <c r="A556" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B556" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C556" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D556" s="2" t="inlineStr">
+        <is>
+          <t>MT373</t>
+        </is>
+      </c>
+      <c r="E556" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F556" s="3" t="n">
+        <v>235500</v>
+      </c>
+      <c r="G556" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="557">
+      <c r="A557" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B557" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C557" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D557" s="2" t="inlineStr">
+        <is>
+          <t>MT374</t>
+        </is>
+      </c>
+      <c r="E557" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F557" s="3" t="n">
+        <v>259500</v>
+      </c>
+      <c r="G557" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="558">
+      <c r="A558" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B558" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C558" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D558" s="2" t="inlineStr">
+        <is>
+          <t>MT375</t>
+        </is>
+      </c>
+      <c r="E558" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F558" s="3" t="n">
+        <v>285500</v>
+      </c>
+      <c r="G558" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="559">
+      <c r="A559" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B559" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C559" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D559" s="2" t="inlineStr">
+        <is>
+          <t>MT376</t>
+        </is>
+      </c>
+      <c r="E559" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F559" s="3" t="n">
+        <v>339500</v>
+      </c>
+      <c r="G559" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="560">
+      <c r="A560" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B560" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C560" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D560" s="2" t="inlineStr">
+        <is>
+          <t>MTY69</t>
+        </is>
+      </c>
+      <c r="E560" s="2" t="inlineStr">
+        <is>
+          <t>Model Y L</t>
+        </is>
+      </c>
+      <c r="F560" s="3" t="n">
+        <v>339000</v>
+      </c>
+      <c r="G560" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="561">
+      <c r="A561" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B561" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C561" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D561" s="2" t="inlineStr">
+        <is>
+          <t>MTY79</t>
+        </is>
+      </c>
+      <c r="E561" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F561" s="3" t="n">
+        <v>263500</v>
+      </c>
+      <c r="G561" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="562">
+      <c r="A562" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B562" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C562" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D562" s="2" t="inlineStr">
+        <is>
+          <t>MTY80</t>
+        </is>
+      </c>
+      <c r="E562" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F562" s="3" t="n">
+        <v>313500</v>
+      </c>
+      <c r="G562" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="563">
+      <c r="A563" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B563" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C563" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D563" s="2" t="inlineStr">
+        <is>
+          <t>MTY81</t>
+        </is>
+      </c>
+      <c r="E563" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F563" s="3" t="n">
+        <v>288500</v>
+      </c>
+      <c r="G563" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="564">
+      <c r="A564" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B564" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C564" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D564" s="2" t="inlineStr">
+        <is>
+          <t>MTY88</t>
+        </is>
+      </c>
+      <c r="E564" s="2" t="inlineStr">
+        <is>
+          <t>Model Y Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F564" s="3" t="n">
+        <v>369000</v>
+      </c>
+      <c r="G564" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price pull 2026-09-30
</commit_message>
<xml_diff>
--- a/tesla_price_analysis.xlsx
+++ b/tesla_price_analysis.xlsx
@@ -445,7 +445,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Snapshot date: 2026-09-29  (source: tesla.com configurator pages)</t>
+          <t>Snapshot date: 2026-09-30  (source: tesla.com configurator pages)</t>
         </is>
       </c>
       <c r="B1" s="1" t="n"/>
@@ -775,7 +775,7 @@
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="19" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -859,7 +859,7 @@
         <v>301125</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>310677.7777777778</v>
+        <v>310821.4285714286</v>
       </c>
     </row>
   </sheetData>
@@ -971,7 +971,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G564"/>
+  <dimension ref="A1:G573"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -20725,6 +20725,321 @@
         </is>
       </c>
     </row>
+    <row r="565">
+      <c r="A565" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B565" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C565" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D565" s="2" t="inlineStr">
+        <is>
+          <t>MT373</t>
+        </is>
+      </c>
+      <c r="E565" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F565" s="3" t="n">
+        <v>235500</v>
+      </c>
+      <c r="G565" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="566">
+      <c r="A566" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B566" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C566" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D566" s="2" t="inlineStr">
+        <is>
+          <t>MT374</t>
+        </is>
+      </c>
+      <c r="E566" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F566" s="3" t="n">
+        <v>259500</v>
+      </c>
+      <c r="G566" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="567">
+      <c r="A567" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B567" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C567" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D567" s="2" t="inlineStr">
+        <is>
+          <t>MT375</t>
+        </is>
+      </c>
+      <c r="E567" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F567" s="3" t="n">
+        <v>285500</v>
+      </c>
+      <c r="G567" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="568">
+      <c r="A568" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B568" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C568" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D568" s="2" t="inlineStr">
+        <is>
+          <t>MT376</t>
+        </is>
+      </c>
+      <c r="E568" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F568" s="3" t="n">
+        <v>339500</v>
+      </c>
+      <c r="G568" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="569">
+      <c r="A569" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B569" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C569" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D569" s="2" t="inlineStr">
+        <is>
+          <t>MTY69</t>
+        </is>
+      </c>
+      <c r="E569" s="2" t="inlineStr">
+        <is>
+          <t>Model Y L</t>
+        </is>
+      </c>
+      <c r="F569" s="3" t="n">
+        <v>339000</v>
+      </c>
+      <c r="G569" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="570">
+      <c r="A570" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B570" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C570" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D570" s="2" t="inlineStr">
+        <is>
+          <t>MTY79</t>
+        </is>
+      </c>
+      <c r="E570" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F570" s="3" t="n">
+        <v>263500</v>
+      </c>
+      <c r="G570" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="571">
+      <c r="A571" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B571" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C571" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D571" s="2" t="inlineStr">
+        <is>
+          <t>MTY80</t>
+        </is>
+      </c>
+      <c r="E571" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F571" s="3" t="n">
+        <v>313500</v>
+      </c>
+      <c r="G571" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="572">
+      <c r="A572" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B572" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C572" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D572" s="2" t="inlineStr">
+        <is>
+          <t>MTY81</t>
+        </is>
+      </c>
+      <c r="E572" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F572" s="3" t="n">
+        <v>288500</v>
+      </c>
+      <c r="G572" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="573">
+      <c r="A573" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B573" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C573" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D573" s="2" t="inlineStr">
+        <is>
+          <t>MTY88</t>
+        </is>
+      </c>
+      <c r="E573" s="2" t="inlineStr">
+        <is>
+          <t>Model Y Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F573" s="3" t="n">
+        <v>369000</v>
+      </c>
+      <c r="G573" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price pull 2026-10-01
</commit_message>
<xml_diff>
--- a/tesla_price_analysis.xlsx
+++ b/tesla_price_analysis.xlsx
@@ -445,7 +445,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Snapshot date: 2026-09-30  (source: tesla.com configurator pages)</t>
+          <t>Snapshot date: 2026-10-01  (source: tesla.com configurator pages)</t>
         </is>
       </c>
       <c r="B1" s="1" t="n"/>
@@ -504,7 +504,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>MT373</t>
+          <t>MT382</t>
         </is>
       </c>
       <c r="E3" s="3" t="n">
@@ -534,7 +534,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>MT374</t>
+          <t>MT383</t>
         </is>
       </c>
       <c r="E4" s="3" t="n">
@@ -564,7 +564,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>MT375</t>
+          <t>MT384</t>
         </is>
       </c>
       <c r="E5" s="3" t="n">
@@ -594,7 +594,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>MT376</t>
+          <t>MT380</t>
         </is>
       </c>
       <c r="E6" s="3" t="n">
@@ -714,7 +714,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>MTY69</t>
+          <t>MTY87</t>
         </is>
       </c>
       <c r="E10" s="3" t="n">
@@ -767,7 +767,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -776,6 +776,7 @@
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="19" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -809,6 +810,11 @@
           <t>2026-09</t>
         </is>
       </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -835,6 +841,9 @@
       <c r="F2" s="3" t="n">
         <v>280000</v>
       </c>
+      <c r="G2" s="3" t="n">
+        <v>280000</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -860,6 +869,9 @@
       </c>
       <c r="F3" s="3" t="n">
         <v>310821.4285714286</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>314700</v>
       </c>
     </row>
   </sheetData>
@@ -873,7 +885,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -881,6 +893,7 @@
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="40" customWidth="1" min="4" max="4"/>
     <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -909,6 +922,11 @@
           <t>2026-09</t>
         </is>
       </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -934,6 +952,10 @@
         <f>IFERROR('Monthly Averages'!F2/'Monthly Averages'!E2-1,"")</f>
         <v/>
       </c>
+      <c r="F2" s="4">
+        <f>IFERROR('Monthly Averages'!G2/'Monthly Averages'!F2-1,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -957,6 +979,10 @@
       </c>
       <c r="E3" s="4">
         <f>IFERROR('Monthly Averages'!F3/'Monthly Averages'!E3-1,"")</f>
+        <v/>
+      </c>
+      <c r="F3" s="4">
+        <f>IFERROR('Monthly Averages'!G3/'Monthly Averages'!F3-1,"")</f>
         <v/>
       </c>
     </row>
@@ -971,7 +997,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G573"/>
+  <dimension ref="A1:G582"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -21040,6 +21066,321 @@
         </is>
       </c>
     </row>
+    <row r="574">
+      <c r="A574" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B574" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C574" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D574" s="2" t="inlineStr">
+        <is>
+          <t>MT380</t>
+        </is>
+      </c>
+      <c r="E574" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F574" s="3" t="n">
+        <v>339500</v>
+      </c>
+      <c r="G574" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="575">
+      <c r="A575" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B575" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C575" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D575" s="2" t="inlineStr">
+        <is>
+          <t>MT382</t>
+        </is>
+      </c>
+      <c r="E575" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F575" s="3" t="n">
+        <v>235500</v>
+      </c>
+      <c r="G575" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="576">
+      <c r="A576" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B576" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C576" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D576" s="2" t="inlineStr">
+        <is>
+          <t>MT383</t>
+        </is>
+      </c>
+      <c r="E576" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F576" s="3" t="n">
+        <v>259500</v>
+      </c>
+      <c r="G576" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="577">
+      <c r="A577" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B577" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C577" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D577" s="2" t="inlineStr">
+        <is>
+          <t>MT384</t>
+        </is>
+      </c>
+      <c r="E577" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F577" s="3" t="n">
+        <v>285500</v>
+      </c>
+      <c r="G577" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="578">
+      <c r="A578" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B578" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C578" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D578" s="2" t="inlineStr">
+        <is>
+          <t>MTY79</t>
+        </is>
+      </c>
+      <c r="E578" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F578" s="3" t="n">
+        <v>263500</v>
+      </c>
+      <c r="G578" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="579">
+      <c r="A579" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B579" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C579" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D579" s="2" t="inlineStr">
+        <is>
+          <t>MTY80</t>
+        </is>
+      </c>
+      <c r="E579" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F579" s="3" t="n">
+        <v>313500</v>
+      </c>
+      <c r="G579" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="580">
+      <c r="A580" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B580" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C580" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D580" s="2" t="inlineStr">
+        <is>
+          <t>MTY81</t>
+        </is>
+      </c>
+      <c r="E580" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F580" s="3" t="n">
+        <v>288500</v>
+      </c>
+      <c r="G580" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="581">
+      <c r="A581" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B581" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C581" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D581" s="2" t="inlineStr">
+        <is>
+          <t>MTY87</t>
+        </is>
+      </c>
+      <c r="E581" s="2" t="inlineStr">
+        <is>
+          <t>Model Y L</t>
+        </is>
+      </c>
+      <c r="F581" s="3" t="n">
+        <v>339000</v>
+      </c>
+      <c r="G581" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="582">
+      <c r="A582" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B582" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C582" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D582" s="2" t="inlineStr">
+        <is>
+          <t>MTY88</t>
+        </is>
+      </c>
+      <c r="E582" s="2" t="inlineStr">
+        <is>
+          <t>Model Y Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F582" s="3" t="n">
+        <v>369000</v>
+      </c>
+      <c r="G582" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price pull 2026-10-02
</commit_message>
<xml_diff>
--- a/tesla_price_analysis.xlsx
+++ b/tesla_price_analysis.xlsx
@@ -445,7 +445,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Snapshot date: 2026-10-01  (source: tesla.com configurator pages)</t>
+          <t>Snapshot date: 2026-10-02  (source: tesla.com configurator pages)</t>
         </is>
       </c>
       <c r="B1" s="1" t="n"/>
@@ -997,7 +997,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G582"/>
+  <dimension ref="A1:G591"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -21381,6 +21381,321 @@
         </is>
       </c>
     </row>
+    <row r="583">
+      <c r="A583" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B583" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C583" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D583" s="2" t="inlineStr">
+        <is>
+          <t>MT380</t>
+        </is>
+      </c>
+      <c r="E583" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F583" s="3" t="n">
+        <v>339500</v>
+      </c>
+      <c r="G583" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="584">
+      <c r="A584" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B584" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C584" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D584" s="2" t="inlineStr">
+        <is>
+          <t>MT382</t>
+        </is>
+      </c>
+      <c r="E584" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F584" s="3" t="n">
+        <v>235500</v>
+      </c>
+      <c r="G584" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="585">
+      <c r="A585" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B585" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C585" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D585" s="2" t="inlineStr">
+        <is>
+          <t>MT383</t>
+        </is>
+      </c>
+      <c r="E585" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F585" s="3" t="n">
+        <v>259500</v>
+      </c>
+      <c r="G585" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="586">
+      <c r="A586" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B586" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C586" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D586" s="2" t="inlineStr">
+        <is>
+          <t>MT384</t>
+        </is>
+      </c>
+      <c r="E586" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F586" s="3" t="n">
+        <v>285500</v>
+      </c>
+      <c r="G586" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="587">
+      <c r="A587" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B587" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C587" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D587" s="2" t="inlineStr">
+        <is>
+          <t>MTY79</t>
+        </is>
+      </c>
+      <c r="E587" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F587" s="3" t="n">
+        <v>263500</v>
+      </c>
+      <c r="G587" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="588">
+      <c r="A588" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B588" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C588" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D588" s="2" t="inlineStr">
+        <is>
+          <t>MTY80</t>
+        </is>
+      </c>
+      <c r="E588" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F588" s="3" t="n">
+        <v>313500</v>
+      </c>
+      <c r="G588" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="589">
+      <c r="A589" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B589" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C589" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D589" s="2" t="inlineStr">
+        <is>
+          <t>MTY81</t>
+        </is>
+      </c>
+      <c r="E589" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F589" s="3" t="n">
+        <v>288500</v>
+      </c>
+      <c r="G589" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="590">
+      <c r="A590" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B590" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C590" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D590" s="2" t="inlineStr">
+        <is>
+          <t>MTY87</t>
+        </is>
+      </c>
+      <c r="E590" s="2" t="inlineStr">
+        <is>
+          <t>Model Y L</t>
+        </is>
+      </c>
+      <c r="F590" s="3" t="n">
+        <v>339000</v>
+      </c>
+      <c r="G590" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="591">
+      <c r="A591" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B591" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C591" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D591" s="2" t="inlineStr">
+        <is>
+          <t>MTY88</t>
+        </is>
+      </c>
+      <c r="E591" s="2" t="inlineStr">
+        <is>
+          <t>Model Y Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F591" s="3" t="n">
+        <v>369000</v>
+      </c>
+      <c r="G591" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price pull 2026-10-03
</commit_message>
<xml_diff>
--- a/tesla_price_analysis.xlsx
+++ b/tesla_price_analysis.xlsx
@@ -445,7 +445,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Snapshot date: 2026-10-02  (source: tesla.com configurator pages)</t>
+          <t>Snapshot date: 2026-10-03  (source: tesla.com configurator pages)</t>
         </is>
       </c>
       <c r="B1" s="1" t="n"/>
@@ -997,7 +997,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G591"/>
+  <dimension ref="A1:G600"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -21696,6 +21696,321 @@
         </is>
       </c>
     </row>
+    <row r="592">
+      <c r="A592" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B592" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C592" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D592" s="2" t="inlineStr">
+        <is>
+          <t>MT380</t>
+        </is>
+      </c>
+      <c r="E592" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F592" s="3" t="n">
+        <v>339500</v>
+      </c>
+      <c r="G592" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="593">
+      <c r="A593" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B593" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C593" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D593" s="2" t="inlineStr">
+        <is>
+          <t>MT382</t>
+        </is>
+      </c>
+      <c r="E593" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F593" s="3" t="n">
+        <v>235500</v>
+      </c>
+      <c r="G593" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="594">
+      <c r="A594" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B594" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C594" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D594" s="2" t="inlineStr">
+        <is>
+          <t>MT383</t>
+        </is>
+      </c>
+      <c r="E594" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F594" s="3" t="n">
+        <v>259500</v>
+      </c>
+      <c r="G594" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="595">
+      <c r="A595" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B595" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C595" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D595" s="2" t="inlineStr">
+        <is>
+          <t>MT384</t>
+        </is>
+      </c>
+      <c r="E595" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F595" s="3" t="n">
+        <v>285500</v>
+      </c>
+      <c r="G595" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="596">
+      <c r="A596" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B596" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C596" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D596" s="2" t="inlineStr">
+        <is>
+          <t>MTY79</t>
+        </is>
+      </c>
+      <c r="E596" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F596" s="3" t="n">
+        <v>263500</v>
+      </c>
+      <c r="G596" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="597">
+      <c r="A597" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B597" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C597" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D597" s="2" t="inlineStr">
+        <is>
+          <t>MTY80</t>
+        </is>
+      </c>
+      <c r="E597" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F597" s="3" t="n">
+        <v>313500</v>
+      </c>
+      <c r="G597" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="598">
+      <c r="A598" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B598" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C598" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D598" s="2" t="inlineStr">
+        <is>
+          <t>MTY81</t>
+        </is>
+      </c>
+      <c r="E598" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F598" s="3" t="n">
+        <v>288500</v>
+      </c>
+      <c r="G598" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="599">
+      <c r="A599" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B599" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C599" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D599" s="2" t="inlineStr">
+        <is>
+          <t>MTY87</t>
+        </is>
+      </c>
+      <c r="E599" s="2" t="inlineStr">
+        <is>
+          <t>Model Y L</t>
+        </is>
+      </c>
+      <c r="F599" s="3" t="n">
+        <v>339000</v>
+      </c>
+      <c r="G599" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="600">
+      <c r="A600" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B600" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C600" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D600" s="2" t="inlineStr">
+        <is>
+          <t>MTY88</t>
+        </is>
+      </c>
+      <c r="E600" s="2" t="inlineStr">
+        <is>
+          <t>Model Y Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F600" s="3" t="n">
+        <v>369000</v>
+      </c>
+      <c r="G600" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price pull 2026-10-04
</commit_message>
<xml_diff>
--- a/tesla_price_analysis.xlsx
+++ b/tesla_price_analysis.xlsx
@@ -445,7 +445,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Snapshot date: 2026-10-03  (source: tesla.com configurator pages)</t>
+          <t>Snapshot date: 2026-10-04  (source: tesla.com configurator pages)</t>
         </is>
       </c>
       <c r="B1" s="1" t="n"/>
@@ -997,7 +997,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G600"/>
+  <dimension ref="A1:G609"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -22011,6 +22011,321 @@
         </is>
       </c>
     </row>
+    <row r="601">
+      <c r="A601" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B601" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C601" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D601" s="2" t="inlineStr">
+        <is>
+          <t>MT380</t>
+        </is>
+      </c>
+      <c r="E601" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F601" s="3" t="n">
+        <v>339500</v>
+      </c>
+      <c r="G601" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="602">
+      <c r="A602" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B602" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C602" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D602" s="2" t="inlineStr">
+        <is>
+          <t>MT382</t>
+        </is>
+      </c>
+      <c r="E602" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F602" s="3" t="n">
+        <v>235500</v>
+      </c>
+      <c r="G602" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="603">
+      <c r="A603" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B603" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C603" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D603" s="2" t="inlineStr">
+        <is>
+          <t>MT383</t>
+        </is>
+      </c>
+      <c r="E603" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F603" s="3" t="n">
+        <v>259500</v>
+      </c>
+      <c r="G603" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="604">
+      <c r="A604" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B604" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C604" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D604" s="2" t="inlineStr">
+        <is>
+          <t>MT384</t>
+        </is>
+      </c>
+      <c r="E604" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F604" s="3" t="n">
+        <v>285500</v>
+      </c>
+      <c r="G604" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="605">
+      <c r="A605" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B605" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C605" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D605" s="2" t="inlineStr">
+        <is>
+          <t>MTY79</t>
+        </is>
+      </c>
+      <c r="E605" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F605" s="3" t="n">
+        <v>263500</v>
+      </c>
+      <c r="G605" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="606">
+      <c r="A606" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B606" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C606" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D606" s="2" t="inlineStr">
+        <is>
+          <t>MTY80</t>
+        </is>
+      </c>
+      <c r="E606" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F606" s="3" t="n">
+        <v>313500</v>
+      </c>
+      <c r="G606" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="607">
+      <c r="A607" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B607" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C607" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D607" s="2" t="inlineStr">
+        <is>
+          <t>MTY81</t>
+        </is>
+      </c>
+      <c r="E607" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F607" s="3" t="n">
+        <v>288500</v>
+      </c>
+      <c r="G607" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="608">
+      <c r="A608" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B608" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C608" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D608" s="2" t="inlineStr">
+        <is>
+          <t>MTY87</t>
+        </is>
+      </c>
+      <c r="E608" s="2" t="inlineStr">
+        <is>
+          <t>Model Y L</t>
+        </is>
+      </c>
+      <c r="F608" s="3" t="n">
+        <v>339000</v>
+      </c>
+      <c r="G608" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="609">
+      <c r="A609" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B609" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C609" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D609" s="2" t="inlineStr">
+        <is>
+          <t>MTY88</t>
+        </is>
+      </c>
+      <c r="E609" s="2" t="inlineStr">
+        <is>
+          <t>Model Y Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F609" s="3" t="n">
+        <v>369000</v>
+      </c>
+      <c r="G609" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price pull 2026-10-05
</commit_message>
<xml_diff>
--- a/tesla_price_analysis.xlsx
+++ b/tesla_price_analysis.xlsx
@@ -445,7 +445,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Snapshot date: 2026-10-04  (source: tesla.com configurator pages)</t>
+          <t>Snapshot date: 2026-10-05  (source: tesla.com configurator pages)</t>
         </is>
       </c>
       <c r="B1" s="1" t="n"/>
@@ -997,7 +997,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G609"/>
+  <dimension ref="A1:G618"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -22326,6 +22326,321 @@
         </is>
       </c>
     </row>
+    <row r="610">
+      <c r="A610" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B610" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C610" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D610" s="2" t="inlineStr">
+        <is>
+          <t>MT380</t>
+        </is>
+      </c>
+      <c r="E610" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F610" s="3" t="n">
+        <v>339500</v>
+      </c>
+      <c r="G610" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="611">
+      <c r="A611" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B611" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C611" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D611" s="2" t="inlineStr">
+        <is>
+          <t>MT382</t>
+        </is>
+      </c>
+      <c r="E611" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F611" s="3" t="n">
+        <v>235500</v>
+      </c>
+      <c r="G611" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="612">
+      <c r="A612" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B612" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C612" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D612" s="2" t="inlineStr">
+        <is>
+          <t>MT383</t>
+        </is>
+      </c>
+      <c r="E612" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F612" s="3" t="n">
+        <v>259500</v>
+      </c>
+      <c r="G612" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="613">
+      <c r="A613" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B613" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C613" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D613" s="2" t="inlineStr">
+        <is>
+          <t>MT384</t>
+        </is>
+      </c>
+      <c r="E613" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F613" s="3" t="n">
+        <v>285500</v>
+      </c>
+      <c r="G613" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="614">
+      <c r="A614" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B614" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C614" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D614" s="2" t="inlineStr">
+        <is>
+          <t>MTY79</t>
+        </is>
+      </c>
+      <c r="E614" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F614" s="3" t="n">
+        <v>263500</v>
+      </c>
+      <c r="G614" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="615">
+      <c r="A615" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B615" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C615" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D615" s="2" t="inlineStr">
+        <is>
+          <t>MTY80</t>
+        </is>
+      </c>
+      <c r="E615" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F615" s="3" t="n">
+        <v>313500</v>
+      </c>
+      <c r="G615" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="616">
+      <c r="A616" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B616" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C616" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D616" s="2" t="inlineStr">
+        <is>
+          <t>MTY81</t>
+        </is>
+      </c>
+      <c r="E616" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F616" s="3" t="n">
+        <v>288500</v>
+      </c>
+      <c r="G616" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="617">
+      <c r="A617" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B617" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C617" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D617" s="2" t="inlineStr">
+        <is>
+          <t>MTY87</t>
+        </is>
+      </c>
+      <c r="E617" s="2" t="inlineStr">
+        <is>
+          <t>Model Y L</t>
+        </is>
+      </c>
+      <c r="F617" s="3" t="n">
+        <v>339000</v>
+      </c>
+      <c r="G617" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="618">
+      <c r="A618" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B618" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C618" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D618" s="2" t="inlineStr">
+        <is>
+          <t>MTY88</t>
+        </is>
+      </c>
+      <c r="E618" s="2" t="inlineStr">
+        <is>
+          <t>Model Y Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F618" s="3" t="n">
+        <v>369000</v>
+      </c>
+      <c r="G618" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price pull 2026-10-06
</commit_message>
<xml_diff>
--- a/tesla_price_analysis.xlsx
+++ b/tesla_price_analysis.xlsx
@@ -445,7 +445,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Snapshot date: 2026-10-05  (source: tesla.com configurator pages)</t>
+          <t>Snapshot date: 2026-10-06  (source: tesla.com configurator pages)</t>
         </is>
       </c>
       <c r="B1" s="1" t="n"/>
@@ -997,7 +997,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G618"/>
+  <dimension ref="A1:G627"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -22641,6 +22641,321 @@
         </is>
       </c>
     </row>
+    <row r="619">
+      <c r="A619" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B619" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C619" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D619" s="2" t="inlineStr">
+        <is>
+          <t>MT380</t>
+        </is>
+      </c>
+      <c r="E619" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F619" s="3" t="n">
+        <v>339500</v>
+      </c>
+      <c r="G619" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="620">
+      <c r="A620" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B620" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C620" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D620" s="2" t="inlineStr">
+        <is>
+          <t>MT382</t>
+        </is>
+      </c>
+      <c r="E620" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F620" s="3" t="n">
+        <v>235500</v>
+      </c>
+      <c r="G620" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="621">
+      <c r="A621" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B621" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C621" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D621" s="2" t="inlineStr">
+        <is>
+          <t>MT383</t>
+        </is>
+      </c>
+      <c r="E621" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F621" s="3" t="n">
+        <v>259500</v>
+      </c>
+      <c r="G621" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="622">
+      <c r="A622" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B622" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C622" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D622" s="2" t="inlineStr">
+        <is>
+          <t>MT384</t>
+        </is>
+      </c>
+      <c r="E622" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F622" s="3" t="n">
+        <v>285500</v>
+      </c>
+      <c r="G622" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="623">
+      <c r="A623" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B623" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C623" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D623" s="2" t="inlineStr">
+        <is>
+          <t>MTY79</t>
+        </is>
+      </c>
+      <c r="E623" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F623" s="3" t="n">
+        <v>263500</v>
+      </c>
+      <c r="G623" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="624">
+      <c r="A624" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B624" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C624" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D624" s="2" t="inlineStr">
+        <is>
+          <t>MTY80</t>
+        </is>
+      </c>
+      <c r="E624" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F624" s="3" t="n">
+        <v>313500</v>
+      </c>
+      <c r="G624" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="625">
+      <c r="A625" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B625" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C625" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D625" s="2" t="inlineStr">
+        <is>
+          <t>MTY81</t>
+        </is>
+      </c>
+      <c r="E625" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F625" s="3" t="n">
+        <v>288500</v>
+      </c>
+      <c r="G625" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="626">
+      <c r="A626" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B626" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C626" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D626" s="2" t="inlineStr">
+        <is>
+          <t>MTY87</t>
+        </is>
+      </c>
+      <c r="E626" s="2" t="inlineStr">
+        <is>
+          <t>Model Y L</t>
+        </is>
+      </c>
+      <c r="F626" s="3" t="n">
+        <v>339000</v>
+      </c>
+      <c r="G626" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="627">
+      <c r="A627" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B627" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C627" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D627" s="2" t="inlineStr">
+        <is>
+          <t>MTY88</t>
+        </is>
+      </c>
+      <c r="E627" s="2" t="inlineStr">
+        <is>
+          <t>Model Y Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F627" s="3" t="n">
+        <v>369000</v>
+      </c>
+      <c r="G627" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price pull 2026-10-07
</commit_message>
<xml_diff>
--- a/tesla_price_analysis.xlsx
+++ b/tesla_price_analysis.xlsx
@@ -445,7 +445,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Snapshot date: 2026-10-06  (source: tesla.com configurator pages)</t>
+          <t>Snapshot date: 2026-10-07  (source: tesla.com configurator pages)</t>
         </is>
       </c>
       <c r="B1" s="1" t="n"/>
@@ -997,7 +997,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G627"/>
+  <dimension ref="A1:G636"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -22956,6 +22956,321 @@
         </is>
       </c>
     </row>
+    <row r="628">
+      <c r="A628" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B628" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C628" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D628" s="2" t="inlineStr">
+        <is>
+          <t>MT380</t>
+        </is>
+      </c>
+      <c r="E628" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F628" s="3" t="n">
+        <v>339500</v>
+      </c>
+      <c r="G628" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="629">
+      <c r="A629" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B629" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C629" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D629" s="2" t="inlineStr">
+        <is>
+          <t>MT382</t>
+        </is>
+      </c>
+      <c r="E629" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F629" s="3" t="n">
+        <v>235500</v>
+      </c>
+      <c r="G629" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="630">
+      <c r="A630" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B630" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C630" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D630" s="2" t="inlineStr">
+        <is>
+          <t>MT383</t>
+        </is>
+      </c>
+      <c r="E630" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F630" s="3" t="n">
+        <v>259500</v>
+      </c>
+      <c r="G630" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="631">
+      <c r="A631" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B631" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C631" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D631" s="2" t="inlineStr">
+        <is>
+          <t>MT384</t>
+        </is>
+      </c>
+      <c r="E631" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F631" s="3" t="n">
+        <v>285500</v>
+      </c>
+      <c r="G631" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="632">
+      <c r="A632" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B632" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C632" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D632" s="2" t="inlineStr">
+        <is>
+          <t>MTY79</t>
+        </is>
+      </c>
+      <c r="E632" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F632" s="3" t="n">
+        <v>263500</v>
+      </c>
+      <c r="G632" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="633">
+      <c r="A633" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B633" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C633" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D633" s="2" t="inlineStr">
+        <is>
+          <t>MTY80</t>
+        </is>
+      </c>
+      <c r="E633" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F633" s="3" t="n">
+        <v>313500</v>
+      </c>
+      <c r="G633" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="634">
+      <c r="A634" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B634" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C634" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D634" s="2" t="inlineStr">
+        <is>
+          <t>MTY81</t>
+        </is>
+      </c>
+      <c r="E634" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F634" s="3" t="n">
+        <v>288500</v>
+      </c>
+      <c r="G634" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="635">
+      <c r="A635" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B635" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C635" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D635" s="2" t="inlineStr">
+        <is>
+          <t>MTY87</t>
+        </is>
+      </c>
+      <c r="E635" s="2" t="inlineStr">
+        <is>
+          <t>Model Y L</t>
+        </is>
+      </c>
+      <c r="F635" s="3" t="n">
+        <v>339000</v>
+      </c>
+      <c r="G635" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="636">
+      <c r="A636" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B636" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C636" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D636" s="2" t="inlineStr">
+        <is>
+          <t>MTY88</t>
+        </is>
+      </c>
+      <c r="E636" s="2" t="inlineStr">
+        <is>
+          <t>Model Y Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F636" s="3" t="n">
+        <v>369000</v>
+      </c>
+      <c r="G636" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price pull 2026-10-08
</commit_message>
<xml_diff>
--- a/tesla_price_analysis.xlsx
+++ b/tesla_price_analysis.xlsx
@@ -445,7 +445,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Snapshot date: 2026-10-07  (source: tesla.com configurator pages)</t>
+          <t>Snapshot date: 2026-10-08  (source: tesla.com configurator pages)</t>
         </is>
       </c>
       <c r="B1" s="1" t="n"/>
@@ -997,7 +997,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G636"/>
+  <dimension ref="A1:G645"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -23271,6 +23271,321 @@
         </is>
       </c>
     </row>
+    <row r="637">
+      <c r="A637" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B637" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C637" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D637" s="2" t="inlineStr">
+        <is>
+          <t>MT380</t>
+        </is>
+      </c>
+      <c r="E637" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F637" s="3" t="n">
+        <v>339500</v>
+      </c>
+      <c r="G637" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="638">
+      <c r="A638" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B638" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C638" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D638" s="2" t="inlineStr">
+        <is>
+          <t>MT382</t>
+        </is>
+      </c>
+      <c r="E638" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F638" s="3" t="n">
+        <v>235500</v>
+      </c>
+      <c r="G638" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="639">
+      <c r="A639" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B639" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C639" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D639" s="2" t="inlineStr">
+        <is>
+          <t>MT383</t>
+        </is>
+      </c>
+      <c r="E639" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F639" s="3" t="n">
+        <v>259500</v>
+      </c>
+      <c r="G639" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="640">
+      <c r="A640" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B640" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C640" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D640" s="2" t="inlineStr">
+        <is>
+          <t>MT384</t>
+        </is>
+      </c>
+      <c r="E640" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F640" s="3" t="n">
+        <v>285500</v>
+      </c>
+      <c r="G640" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="641">
+      <c r="A641" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B641" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C641" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D641" s="2" t="inlineStr">
+        <is>
+          <t>MTY79</t>
+        </is>
+      </c>
+      <c r="E641" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F641" s="3" t="n">
+        <v>263500</v>
+      </c>
+      <c r="G641" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="642">
+      <c r="A642" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B642" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C642" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D642" s="2" t="inlineStr">
+        <is>
+          <t>MTY80</t>
+        </is>
+      </c>
+      <c r="E642" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F642" s="3" t="n">
+        <v>313500</v>
+      </c>
+      <c r="G642" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="643">
+      <c r="A643" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B643" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C643" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D643" s="2" t="inlineStr">
+        <is>
+          <t>MTY81</t>
+        </is>
+      </c>
+      <c r="E643" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F643" s="3" t="n">
+        <v>288500</v>
+      </c>
+      <c r="G643" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="644">
+      <c r="A644" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B644" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C644" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D644" s="2" t="inlineStr">
+        <is>
+          <t>MTY87</t>
+        </is>
+      </c>
+      <c r="E644" s="2" t="inlineStr">
+        <is>
+          <t>Model Y L</t>
+        </is>
+      </c>
+      <c r="F644" s="3" t="n">
+        <v>339000</v>
+      </c>
+      <c r="G644" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="645">
+      <c r="A645" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B645" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C645" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D645" s="2" t="inlineStr">
+        <is>
+          <t>MTY88</t>
+        </is>
+      </c>
+      <c r="E645" s="2" t="inlineStr">
+        <is>
+          <t>Model Y Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F645" s="3" t="n">
+        <v>369000</v>
+      </c>
+      <c r="G645" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price pull 2026-10-09
</commit_message>
<xml_diff>
--- a/tesla_price_analysis.xlsx
+++ b/tesla_price_analysis.xlsx
@@ -445,7 +445,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Snapshot date: 2026-10-08  (source: tesla.com configurator pages)</t>
+          <t>Snapshot date: 2026-10-09  (source: tesla.com configurator pages)</t>
         </is>
       </c>
       <c r="B1" s="1" t="n"/>
@@ -997,7 +997,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G645"/>
+  <dimension ref="A1:G654"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -23586,6 +23586,321 @@
         </is>
       </c>
     </row>
+    <row r="646">
+      <c r="A646" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B646" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C646" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D646" s="2" t="inlineStr">
+        <is>
+          <t>MT380</t>
+        </is>
+      </c>
+      <c r="E646" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F646" s="3" t="n">
+        <v>339500</v>
+      </c>
+      <c r="G646" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="647">
+      <c r="A647" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B647" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C647" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D647" s="2" t="inlineStr">
+        <is>
+          <t>MT382</t>
+        </is>
+      </c>
+      <c r="E647" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F647" s="3" t="n">
+        <v>235500</v>
+      </c>
+      <c r="G647" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="648">
+      <c r="A648" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B648" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C648" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D648" s="2" t="inlineStr">
+        <is>
+          <t>MT383</t>
+        </is>
+      </c>
+      <c r="E648" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F648" s="3" t="n">
+        <v>259500</v>
+      </c>
+      <c r="G648" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="649">
+      <c r="A649" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B649" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C649" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D649" s="2" t="inlineStr">
+        <is>
+          <t>MT384</t>
+        </is>
+      </c>
+      <c r="E649" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F649" s="3" t="n">
+        <v>285500</v>
+      </c>
+      <c r="G649" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="650">
+      <c r="A650" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B650" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C650" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D650" s="2" t="inlineStr">
+        <is>
+          <t>MTY79</t>
+        </is>
+      </c>
+      <c r="E650" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F650" s="3" t="n">
+        <v>263500</v>
+      </c>
+      <c r="G650" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="651">
+      <c r="A651" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B651" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C651" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D651" s="2" t="inlineStr">
+        <is>
+          <t>MTY80</t>
+        </is>
+      </c>
+      <c r="E651" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F651" s="3" t="n">
+        <v>313500</v>
+      </c>
+      <c r="G651" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="652">
+      <c r="A652" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B652" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C652" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D652" s="2" t="inlineStr">
+        <is>
+          <t>MTY81</t>
+        </is>
+      </c>
+      <c r="E652" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F652" s="3" t="n">
+        <v>288500</v>
+      </c>
+      <c r="G652" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="653">
+      <c r="A653" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B653" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C653" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D653" s="2" t="inlineStr">
+        <is>
+          <t>MTY87</t>
+        </is>
+      </c>
+      <c r="E653" s="2" t="inlineStr">
+        <is>
+          <t>Model Y L</t>
+        </is>
+      </c>
+      <c r="F653" s="3" t="n">
+        <v>339000</v>
+      </c>
+      <c r="G653" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="654">
+      <c r="A654" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="B654" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C654" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D654" s="2" t="inlineStr">
+        <is>
+          <t>MTY88</t>
+        </is>
+      </c>
+      <c r="E654" s="2" t="inlineStr">
+        <is>
+          <t>Model Y Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F654" s="3" t="n">
+        <v>369000</v>
+      </c>
+      <c r="G654" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price pull 2026-10-10
</commit_message>
<xml_diff>
--- a/tesla_price_analysis.xlsx
+++ b/tesla_price_analysis.xlsx
@@ -445,7 +445,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Snapshot date: 2026-10-09  (source: tesla.com configurator pages)</t>
+          <t>Snapshot date: 2026-10-10  (source: tesla.com configurator pages)</t>
         </is>
       </c>
       <c r="B1" s="1" t="n"/>
@@ -997,7 +997,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G654"/>
+  <dimension ref="A1:G663"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -23901,6 +23901,321 @@
         </is>
       </c>
     </row>
+    <row r="655">
+      <c r="A655" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B655" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C655" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D655" s="2" t="inlineStr">
+        <is>
+          <t>MT380</t>
+        </is>
+      </c>
+      <c r="E655" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F655" s="3" t="n">
+        <v>339500</v>
+      </c>
+      <c r="G655" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="656">
+      <c r="A656" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B656" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C656" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D656" s="2" t="inlineStr">
+        <is>
+          <t>MT382</t>
+        </is>
+      </c>
+      <c r="E656" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F656" s="3" t="n">
+        <v>235500</v>
+      </c>
+      <c r="G656" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="657">
+      <c r="A657" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B657" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C657" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D657" s="2" t="inlineStr">
+        <is>
+          <t>MT383</t>
+        </is>
+      </c>
+      <c r="E657" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F657" s="3" t="n">
+        <v>259500</v>
+      </c>
+      <c r="G657" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="658">
+      <c r="A658" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B658" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C658" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D658" s="2" t="inlineStr">
+        <is>
+          <t>MT384</t>
+        </is>
+      </c>
+      <c r="E658" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F658" s="3" t="n">
+        <v>285500</v>
+      </c>
+      <c r="G658" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="659">
+      <c r="A659" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B659" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C659" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D659" s="2" t="inlineStr">
+        <is>
+          <t>MTY79</t>
+        </is>
+      </c>
+      <c r="E659" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F659" s="3" t="n">
+        <v>263500</v>
+      </c>
+      <c r="G659" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="660">
+      <c r="A660" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B660" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C660" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D660" s="2" t="inlineStr">
+        <is>
+          <t>MTY80</t>
+        </is>
+      </c>
+      <c r="E660" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F660" s="3" t="n">
+        <v>313500</v>
+      </c>
+      <c r="G660" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="661">
+      <c r="A661" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B661" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C661" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D661" s="2" t="inlineStr">
+        <is>
+          <t>MTY81</t>
+        </is>
+      </c>
+      <c r="E661" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F661" s="3" t="n">
+        <v>288500</v>
+      </c>
+      <c r="G661" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="662">
+      <c r="A662" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B662" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C662" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D662" s="2" t="inlineStr">
+        <is>
+          <t>MTY87</t>
+        </is>
+      </c>
+      <c r="E662" s="2" t="inlineStr">
+        <is>
+          <t>Model Y L</t>
+        </is>
+      </c>
+      <c r="F662" s="3" t="n">
+        <v>339000</v>
+      </c>
+      <c r="G662" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="663">
+      <c r="A663" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B663" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C663" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D663" s="2" t="inlineStr">
+        <is>
+          <t>MTY88</t>
+        </is>
+      </c>
+      <c r="E663" s="2" t="inlineStr">
+        <is>
+          <t>Model Y Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F663" s="3" t="n">
+        <v>369000</v>
+      </c>
+      <c r="G663" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price pull 2026-10-11
</commit_message>
<xml_diff>
--- a/tesla_price_analysis.xlsx
+++ b/tesla_price_analysis.xlsx
@@ -445,7 +445,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Snapshot date: 2026-10-10  (source: tesla.com configurator pages)</t>
+          <t>Snapshot date: 2026-10-11  (source: tesla.com configurator pages)</t>
         </is>
       </c>
       <c r="B1" s="1" t="n"/>
@@ -997,7 +997,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G663"/>
+  <dimension ref="A1:G672"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -24216,6 +24216,321 @@
         </is>
       </c>
     </row>
+    <row r="664">
+      <c r="A664" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B664" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C664" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D664" s="2" t="inlineStr">
+        <is>
+          <t>MT380</t>
+        </is>
+      </c>
+      <c r="E664" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F664" s="3" t="n">
+        <v>339500</v>
+      </c>
+      <c r="G664" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="665">
+      <c r="A665" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B665" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C665" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D665" s="2" t="inlineStr">
+        <is>
+          <t>MT382</t>
+        </is>
+      </c>
+      <c r="E665" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F665" s="3" t="n">
+        <v>235500</v>
+      </c>
+      <c r="G665" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="666">
+      <c r="A666" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B666" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C666" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D666" s="2" t="inlineStr">
+        <is>
+          <t>MT383</t>
+        </is>
+      </c>
+      <c r="E666" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F666" s="3" t="n">
+        <v>259500</v>
+      </c>
+      <c r="G666" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="667">
+      <c r="A667" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B667" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C667" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D667" s="2" t="inlineStr">
+        <is>
+          <t>MT384</t>
+        </is>
+      </c>
+      <c r="E667" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F667" s="3" t="n">
+        <v>285500</v>
+      </c>
+      <c r="G667" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="668">
+      <c r="A668" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B668" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C668" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D668" s="2" t="inlineStr">
+        <is>
+          <t>MTY79</t>
+        </is>
+      </c>
+      <c r="E668" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F668" s="3" t="n">
+        <v>263500</v>
+      </c>
+      <c r="G668" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="669">
+      <c r="A669" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B669" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C669" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D669" s="2" t="inlineStr">
+        <is>
+          <t>MTY80</t>
+        </is>
+      </c>
+      <c r="E669" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F669" s="3" t="n">
+        <v>313500</v>
+      </c>
+      <c r="G669" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="670">
+      <c r="A670" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B670" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C670" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D670" s="2" t="inlineStr">
+        <is>
+          <t>MTY81</t>
+        </is>
+      </c>
+      <c r="E670" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F670" s="3" t="n">
+        <v>288500</v>
+      </c>
+      <c r="G670" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="671">
+      <c r="A671" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B671" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C671" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D671" s="2" t="inlineStr">
+        <is>
+          <t>MTY87</t>
+        </is>
+      </c>
+      <c r="E671" s="2" t="inlineStr">
+        <is>
+          <t>Model Y L</t>
+        </is>
+      </c>
+      <c r="F671" s="3" t="n">
+        <v>339000</v>
+      </c>
+      <c r="G671" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="672">
+      <c r="A672" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B672" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C672" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D672" s="2" t="inlineStr">
+        <is>
+          <t>MTY88</t>
+        </is>
+      </c>
+      <c r="E672" s="2" t="inlineStr">
+        <is>
+          <t>Model Y Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F672" s="3" t="n">
+        <v>369000</v>
+      </c>
+      <c r="G672" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price pull 2026-10-12
</commit_message>
<xml_diff>
--- a/tesla_price_analysis.xlsx
+++ b/tesla_price_analysis.xlsx
@@ -445,7 +445,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Snapshot date: 2026-10-11  (source: tesla.com configurator pages)</t>
+          <t>Snapshot date: 2026-10-12  (source: tesla.com configurator pages)</t>
         </is>
       </c>
       <c r="B1" s="1" t="n"/>
@@ -997,7 +997,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G672"/>
+  <dimension ref="A1:G681"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -24531,6 +24531,321 @@
         </is>
       </c>
     </row>
+    <row r="673">
+      <c r="A673" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B673" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C673" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D673" s="2" t="inlineStr">
+        <is>
+          <t>MT380</t>
+        </is>
+      </c>
+      <c r="E673" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F673" s="3" t="n">
+        <v>339500</v>
+      </c>
+      <c r="G673" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="674">
+      <c r="A674" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B674" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C674" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D674" s="2" t="inlineStr">
+        <is>
+          <t>MT382</t>
+        </is>
+      </c>
+      <c r="E674" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F674" s="3" t="n">
+        <v>235500</v>
+      </c>
+      <c r="G674" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="675">
+      <c r="A675" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B675" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C675" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D675" s="2" t="inlineStr">
+        <is>
+          <t>MT383</t>
+        </is>
+      </c>
+      <c r="E675" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F675" s="3" t="n">
+        <v>259500</v>
+      </c>
+      <c r="G675" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="676">
+      <c r="A676" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B676" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C676" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D676" s="2" t="inlineStr">
+        <is>
+          <t>MT384</t>
+        </is>
+      </c>
+      <c r="E676" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F676" s="3" t="n">
+        <v>285500</v>
+      </c>
+      <c r="G676" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="677">
+      <c r="A677" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B677" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C677" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D677" s="2" t="inlineStr">
+        <is>
+          <t>MTY79</t>
+        </is>
+      </c>
+      <c r="E677" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F677" s="3" t="n">
+        <v>263500</v>
+      </c>
+      <c r="G677" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="678">
+      <c r="A678" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B678" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C678" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D678" s="2" t="inlineStr">
+        <is>
+          <t>MTY80</t>
+        </is>
+      </c>
+      <c r="E678" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F678" s="3" t="n">
+        <v>313500</v>
+      </c>
+      <c r="G678" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="679">
+      <c r="A679" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B679" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C679" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D679" s="2" t="inlineStr">
+        <is>
+          <t>MTY81</t>
+        </is>
+      </c>
+      <c r="E679" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F679" s="3" t="n">
+        <v>288500</v>
+      </c>
+      <c r="G679" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="680">
+      <c r="A680" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B680" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C680" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D680" s="2" t="inlineStr">
+        <is>
+          <t>MTY87</t>
+        </is>
+      </c>
+      <c r="E680" s="2" t="inlineStr">
+        <is>
+          <t>Model Y L</t>
+        </is>
+      </c>
+      <c r="F680" s="3" t="n">
+        <v>339000</v>
+      </c>
+      <c r="G680" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="681">
+      <c r="A681" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B681" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C681" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D681" s="2" t="inlineStr">
+        <is>
+          <t>MTY88</t>
+        </is>
+      </c>
+      <c r="E681" s="2" t="inlineStr">
+        <is>
+          <t>Model Y Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F681" s="3" t="n">
+        <v>369000</v>
+      </c>
+      <c r="G681" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price pull 2026-10-13
</commit_message>
<xml_diff>
--- a/tesla_price_analysis.xlsx
+++ b/tesla_price_analysis.xlsx
@@ -445,7 +445,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Snapshot date: 2026-10-12  (source: tesla.com configurator pages)</t>
+          <t>Snapshot date: 2026-10-13  (source: tesla.com configurator pages)</t>
         </is>
       </c>
       <c r="B1" s="1" t="n"/>
@@ -997,7 +997,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G681"/>
+  <dimension ref="A1:G690"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -24846,6 +24846,321 @@
         </is>
       </c>
     </row>
+    <row r="682">
+      <c r="A682" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B682" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C682" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D682" s="2" t="inlineStr">
+        <is>
+          <t>MT380</t>
+        </is>
+      </c>
+      <c r="E682" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F682" s="3" t="n">
+        <v>339500</v>
+      </c>
+      <c r="G682" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="683">
+      <c r="A683" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B683" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C683" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D683" s="2" t="inlineStr">
+        <is>
+          <t>MT382</t>
+        </is>
+      </c>
+      <c r="E683" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F683" s="3" t="n">
+        <v>235500</v>
+      </c>
+      <c r="G683" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="684">
+      <c r="A684" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B684" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C684" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D684" s="2" t="inlineStr">
+        <is>
+          <t>MT383</t>
+        </is>
+      </c>
+      <c r="E684" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F684" s="3" t="n">
+        <v>259500</v>
+      </c>
+      <c r="G684" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="685">
+      <c r="A685" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B685" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C685" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D685" s="2" t="inlineStr">
+        <is>
+          <t>MT384</t>
+        </is>
+      </c>
+      <c r="E685" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F685" s="3" t="n">
+        <v>285500</v>
+      </c>
+      <c r="G685" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="686">
+      <c r="A686" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B686" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C686" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D686" s="2" t="inlineStr">
+        <is>
+          <t>MTY79</t>
+        </is>
+      </c>
+      <c r="E686" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F686" s="3" t="n">
+        <v>263500</v>
+      </c>
+      <c r="G686" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="687">
+      <c r="A687" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B687" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C687" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D687" s="2" t="inlineStr">
+        <is>
+          <t>MTY80</t>
+        </is>
+      </c>
+      <c r="E687" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F687" s="3" t="n">
+        <v>313500</v>
+      </c>
+      <c r="G687" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="688">
+      <c r="A688" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B688" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C688" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D688" s="2" t="inlineStr">
+        <is>
+          <t>MTY81</t>
+        </is>
+      </c>
+      <c r="E688" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F688" s="3" t="n">
+        <v>288500</v>
+      </c>
+      <c r="G688" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="689">
+      <c r="A689" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B689" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C689" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D689" s="2" t="inlineStr">
+        <is>
+          <t>MTY87</t>
+        </is>
+      </c>
+      <c r="E689" s="2" t="inlineStr">
+        <is>
+          <t>Model Y L</t>
+        </is>
+      </c>
+      <c r="F689" s="3" t="n">
+        <v>339000</v>
+      </c>
+      <c r="G689" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="690">
+      <c r="A690" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B690" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C690" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D690" s="2" t="inlineStr">
+        <is>
+          <t>MTY88</t>
+        </is>
+      </c>
+      <c r="E690" s="2" t="inlineStr">
+        <is>
+          <t>Model Y Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F690" s="3" t="n">
+        <v>369000</v>
+      </c>
+      <c r="G690" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price pull 2026-10-14
</commit_message>
<xml_diff>
--- a/tesla_price_analysis.xlsx
+++ b/tesla_price_analysis.xlsx
@@ -445,7 +445,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Snapshot date: 2026-10-13  (source: tesla.com configurator pages)</t>
+          <t>Snapshot date: 2026-10-14  (source: tesla.com configurator pages)</t>
         </is>
       </c>
       <c r="B1" s="1" t="n"/>
@@ -997,7 +997,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G690"/>
+  <dimension ref="A1:G699"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -25161,6 +25161,321 @@
         </is>
       </c>
     </row>
+    <row r="691">
+      <c r="A691" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B691" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C691" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D691" s="2" t="inlineStr">
+        <is>
+          <t>MT380</t>
+        </is>
+      </c>
+      <c r="E691" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F691" s="3" t="n">
+        <v>339500</v>
+      </c>
+      <c r="G691" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="692">
+      <c r="A692" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B692" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C692" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D692" s="2" t="inlineStr">
+        <is>
+          <t>MT382</t>
+        </is>
+      </c>
+      <c r="E692" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F692" s="3" t="n">
+        <v>235500</v>
+      </c>
+      <c r="G692" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="693">
+      <c r="A693" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B693" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C693" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D693" s="2" t="inlineStr">
+        <is>
+          <t>MT383</t>
+        </is>
+      </c>
+      <c r="E693" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F693" s="3" t="n">
+        <v>259500</v>
+      </c>
+      <c r="G693" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="694">
+      <c r="A694" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B694" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C694" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D694" s="2" t="inlineStr">
+        <is>
+          <t>MT384</t>
+        </is>
+      </c>
+      <c r="E694" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F694" s="3" t="n">
+        <v>285500</v>
+      </c>
+      <c r="G694" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="695">
+      <c r="A695" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B695" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C695" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D695" s="2" t="inlineStr">
+        <is>
+          <t>MTY79</t>
+        </is>
+      </c>
+      <c r="E695" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F695" s="3" t="n">
+        <v>263500</v>
+      </c>
+      <c r="G695" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="696">
+      <c r="A696" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B696" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C696" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D696" s="2" t="inlineStr">
+        <is>
+          <t>MTY80</t>
+        </is>
+      </c>
+      <c r="E696" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F696" s="3" t="n">
+        <v>313500</v>
+      </c>
+      <c r="G696" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="697">
+      <c r="A697" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B697" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C697" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D697" s="2" t="inlineStr">
+        <is>
+          <t>MTY81</t>
+        </is>
+      </c>
+      <c r="E697" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F697" s="3" t="n">
+        <v>288500</v>
+      </c>
+      <c r="G697" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="698">
+      <c r="A698" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B698" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C698" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D698" s="2" t="inlineStr">
+        <is>
+          <t>MTY87</t>
+        </is>
+      </c>
+      <c r="E698" s="2" t="inlineStr">
+        <is>
+          <t>Model Y L</t>
+        </is>
+      </c>
+      <c r="F698" s="3" t="n">
+        <v>339000</v>
+      </c>
+      <c r="G698" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="699">
+      <c r="A699" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B699" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C699" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D699" s="2" t="inlineStr">
+        <is>
+          <t>MTY88</t>
+        </is>
+      </c>
+      <c r="E699" s="2" t="inlineStr">
+        <is>
+          <t>Model Y Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F699" s="3" t="n">
+        <v>369000</v>
+      </c>
+      <c r="G699" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price pull 2026-10-15
</commit_message>
<xml_diff>
--- a/tesla_price_analysis.xlsx
+++ b/tesla_price_analysis.xlsx
@@ -445,7 +445,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Snapshot date: 2026-10-14  (source: tesla.com configurator pages)</t>
+          <t>Snapshot date: 2026-10-15  (source: tesla.com configurator pages)</t>
         </is>
       </c>
       <c r="B1" s="1" t="n"/>
@@ -997,7 +997,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G699"/>
+  <dimension ref="A1:G708"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -25476,6 +25476,321 @@
         </is>
       </c>
     </row>
+    <row r="700">
+      <c r="A700" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B700" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C700" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D700" s="2" t="inlineStr">
+        <is>
+          <t>MT380</t>
+        </is>
+      </c>
+      <c r="E700" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F700" s="3" t="n">
+        <v>339500</v>
+      </c>
+      <c r="G700" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="701">
+      <c r="A701" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B701" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C701" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D701" s="2" t="inlineStr">
+        <is>
+          <t>MT382</t>
+        </is>
+      </c>
+      <c r="E701" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F701" s="3" t="n">
+        <v>235500</v>
+      </c>
+      <c r="G701" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="702">
+      <c r="A702" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B702" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C702" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D702" s="2" t="inlineStr">
+        <is>
+          <t>MT383</t>
+        </is>
+      </c>
+      <c r="E702" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F702" s="3" t="n">
+        <v>259500</v>
+      </c>
+      <c r="G702" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="703">
+      <c r="A703" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B703" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C703" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D703" s="2" t="inlineStr">
+        <is>
+          <t>MT384</t>
+        </is>
+      </c>
+      <c r="E703" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F703" s="3" t="n">
+        <v>285500</v>
+      </c>
+      <c r="G703" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="704">
+      <c r="A704" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B704" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C704" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D704" s="2" t="inlineStr">
+        <is>
+          <t>MTY79</t>
+        </is>
+      </c>
+      <c r="E704" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F704" s="3" t="n">
+        <v>263500</v>
+      </c>
+      <c r="G704" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="705">
+      <c r="A705" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B705" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C705" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D705" s="2" t="inlineStr">
+        <is>
+          <t>MTY80</t>
+        </is>
+      </c>
+      <c r="E705" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F705" s="3" t="n">
+        <v>313500</v>
+      </c>
+      <c r="G705" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="706">
+      <c r="A706" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B706" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C706" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D706" s="2" t="inlineStr">
+        <is>
+          <t>MTY81</t>
+        </is>
+      </c>
+      <c r="E706" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F706" s="3" t="n">
+        <v>288500</v>
+      </c>
+      <c r="G706" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="707">
+      <c r="A707" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B707" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C707" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D707" s="2" t="inlineStr">
+        <is>
+          <t>MTY87</t>
+        </is>
+      </c>
+      <c r="E707" s="2" t="inlineStr">
+        <is>
+          <t>Model Y L</t>
+        </is>
+      </c>
+      <c r="F707" s="3" t="n">
+        <v>339000</v>
+      </c>
+      <c r="G707" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="708">
+      <c r="A708" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B708" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C708" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D708" s="2" t="inlineStr">
+        <is>
+          <t>MTY88</t>
+        </is>
+      </c>
+      <c r="E708" s="2" t="inlineStr">
+        <is>
+          <t>Model Y Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F708" s="3" t="n">
+        <v>369000</v>
+      </c>
+      <c r="G708" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price pull 2026-10-16
</commit_message>
<xml_diff>
--- a/tesla_price_analysis.xlsx
+++ b/tesla_price_analysis.xlsx
@@ -445,7 +445,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Snapshot date: 2026-10-15  (source: tesla.com configurator pages)</t>
+          <t>Snapshot date: 2026-10-16  (source: tesla.com configurator pages)</t>
         </is>
       </c>
       <c r="B1" s="1" t="n"/>
@@ -997,7 +997,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G708"/>
+  <dimension ref="A1:G717"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -25791,6 +25791,321 @@
         </is>
       </c>
     </row>
+    <row r="709">
+      <c r="A709" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B709" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C709" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D709" s="2" t="inlineStr">
+        <is>
+          <t>MT380</t>
+        </is>
+      </c>
+      <c r="E709" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F709" s="3" t="n">
+        <v>339500</v>
+      </c>
+      <c r="G709" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="710">
+      <c r="A710" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B710" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C710" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D710" s="2" t="inlineStr">
+        <is>
+          <t>MT382</t>
+        </is>
+      </c>
+      <c r="E710" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F710" s="3" t="n">
+        <v>235500</v>
+      </c>
+      <c r="G710" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="711">
+      <c r="A711" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B711" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C711" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D711" s="2" t="inlineStr">
+        <is>
+          <t>MT383</t>
+        </is>
+      </c>
+      <c r="E711" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F711" s="3" t="n">
+        <v>259500</v>
+      </c>
+      <c r="G711" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="712">
+      <c r="A712" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B712" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C712" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D712" s="2" t="inlineStr">
+        <is>
+          <t>MT384</t>
+        </is>
+      </c>
+      <c r="E712" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F712" s="3" t="n">
+        <v>285500</v>
+      </c>
+      <c r="G712" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="713">
+      <c r="A713" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B713" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C713" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D713" s="2" t="inlineStr">
+        <is>
+          <t>MTY79</t>
+        </is>
+      </c>
+      <c r="E713" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F713" s="3" t="n">
+        <v>263500</v>
+      </c>
+      <c r="G713" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="714">
+      <c r="A714" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B714" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C714" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D714" s="2" t="inlineStr">
+        <is>
+          <t>MTY80</t>
+        </is>
+      </c>
+      <c r="E714" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F714" s="3" t="n">
+        <v>313500</v>
+      </c>
+      <c r="G714" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="715">
+      <c r="A715" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B715" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C715" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D715" s="2" t="inlineStr">
+        <is>
+          <t>MTY81</t>
+        </is>
+      </c>
+      <c r="E715" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F715" s="3" t="n">
+        <v>288500</v>
+      </c>
+      <c r="G715" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="716">
+      <c r="A716" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B716" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C716" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D716" s="2" t="inlineStr">
+        <is>
+          <t>MTY87</t>
+        </is>
+      </c>
+      <c r="E716" s="2" t="inlineStr">
+        <is>
+          <t>Model Y L</t>
+        </is>
+      </c>
+      <c r="F716" s="3" t="n">
+        <v>339000</v>
+      </c>
+      <c r="G716" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="717">
+      <c r="A717" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B717" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C717" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D717" s="2" t="inlineStr">
+        <is>
+          <t>MTY88</t>
+        </is>
+      </c>
+      <c r="E717" s="2" t="inlineStr">
+        <is>
+          <t>Model Y Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F717" s="3" t="n">
+        <v>369000</v>
+      </c>
+      <c r="G717" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price pull 2026-10-17
</commit_message>
<xml_diff>
--- a/tesla_price_analysis.xlsx
+++ b/tesla_price_analysis.xlsx
@@ -445,7 +445,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Snapshot date: 2026-10-16  (source: tesla.com configurator pages)</t>
+          <t>Snapshot date: 2026-10-17  (source: tesla.com configurator pages)</t>
         </is>
       </c>
       <c r="B1" s="1" t="n"/>
@@ -997,7 +997,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G717"/>
+  <dimension ref="A1:G726"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -26106,6 +26106,321 @@
         </is>
       </c>
     </row>
+    <row r="718">
+      <c r="A718" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B718" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C718" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D718" s="2" t="inlineStr">
+        <is>
+          <t>MT380</t>
+        </is>
+      </c>
+      <c r="E718" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F718" s="3" t="n">
+        <v>339500</v>
+      </c>
+      <c r="G718" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="719">
+      <c r="A719" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B719" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C719" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D719" s="2" t="inlineStr">
+        <is>
+          <t>MT382</t>
+        </is>
+      </c>
+      <c r="E719" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F719" s="3" t="n">
+        <v>235500</v>
+      </c>
+      <c r="G719" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="720">
+      <c r="A720" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B720" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C720" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D720" s="2" t="inlineStr">
+        <is>
+          <t>MT383</t>
+        </is>
+      </c>
+      <c r="E720" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F720" s="3" t="n">
+        <v>259500</v>
+      </c>
+      <c r="G720" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="721">
+      <c r="A721" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B721" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C721" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D721" s="2" t="inlineStr">
+        <is>
+          <t>MT384</t>
+        </is>
+      </c>
+      <c r="E721" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F721" s="3" t="n">
+        <v>285500</v>
+      </c>
+      <c r="G721" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="722">
+      <c r="A722" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B722" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C722" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D722" s="2" t="inlineStr">
+        <is>
+          <t>MTY79</t>
+        </is>
+      </c>
+      <c r="E722" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F722" s="3" t="n">
+        <v>263500</v>
+      </c>
+      <c r="G722" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="723">
+      <c r="A723" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B723" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C723" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D723" s="2" t="inlineStr">
+        <is>
+          <t>MTY80</t>
+        </is>
+      </c>
+      <c r="E723" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F723" s="3" t="n">
+        <v>313500</v>
+      </c>
+      <c r="G723" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="724">
+      <c r="A724" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B724" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C724" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D724" s="2" t="inlineStr">
+        <is>
+          <t>MTY81</t>
+        </is>
+      </c>
+      <c r="E724" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F724" s="3" t="n">
+        <v>288500</v>
+      </c>
+      <c r="G724" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="725">
+      <c r="A725" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B725" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C725" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D725" s="2" t="inlineStr">
+        <is>
+          <t>MTY87</t>
+        </is>
+      </c>
+      <c r="E725" s="2" t="inlineStr">
+        <is>
+          <t>Model Y L</t>
+        </is>
+      </c>
+      <c r="F725" s="3" t="n">
+        <v>339000</v>
+      </c>
+      <c r="G725" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="726">
+      <c r="A726" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B726" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C726" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D726" s="2" t="inlineStr">
+        <is>
+          <t>MTY88</t>
+        </is>
+      </c>
+      <c r="E726" s="2" t="inlineStr">
+        <is>
+          <t>Model Y Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F726" s="3" t="n">
+        <v>369000</v>
+      </c>
+      <c r="G726" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price pull 2026-10-18
</commit_message>
<xml_diff>
--- a/tesla_price_analysis.xlsx
+++ b/tesla_price_analysis.xlsx
@@ -445,7 +445,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Snapshot date: 2026-10-17  (source: tesla.com configurator pages)</t>
+          <t>Snapshot date: 2026-10-18  (source: tesla.com configurator pages)</t>
         </is>
       </c>
       <c r="B1" s="1" t="n"/>
@@ -997,7 +997,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G726"/>
+  <dimension ref="A1:G735"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -26421,6 +26421,321 @@
         </is>
       </c>
     </row>
+    <row r="727">
+      <c r="A727" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B727" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C727" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D727" s="2" t="inlineStr">
+        <is>
+          <t>MT380</t>
+        </is>
+      </c>
+      <c r="E727" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F727" s="3" t="n">
+        <v>339500</v>
+      </c>
+      <c r="G727" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="728">
+      <c r="A728" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B728" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C728" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D728" s="2" t="inlineStr">
+        <is>
+          <t>MT382</t>
+        </is>
+      </c>
+      <c r="E728" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F728" s="3" t="n">
+        <v>235500</v>
+      </c>
+      <c r="G728" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="729">
+      <c r="A729" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B729" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C729" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D729" s="2" t="inlineStr">
+        <is>
+          <t>MT383</t>
+        </is>
+      </c>
+      <c r="E729" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F729" s="3" t="n">
+        <v>259500</v>
+      </c>
+      <c r="G729" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="730">
+      <c r="A730" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B730" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C730" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D730" s="2" t="inlineStr">
+        <is>
+          <t>MT384</t>
+        </is>
+      </c>
+      <c r="E730" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F730" s="3" t="n">
+        <v>285500</v>
+      </c>
+      <c r="G730" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="731">
+      <c r="A731" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B731" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C731" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D731" s="2" t="inlineStr">
+        <is>
+          <t>MTY79</t>
+        </is>
+      </c>
+      <c r="E731" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F731" s="3" t="n">
+        <v>263500</v>
+      </c>
+      <c r="G731" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="732">
+      <c r="A732" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B732" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C732" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D732" s="2" t="inlineStr">
+        <is>
+          <t>MTY80</t>
+        </is>
+      </c>
+      <c r="E732" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F732" s="3" t="n">
+        <v>313500</v>
+      </c>
+      <c r="G732" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="733">
+      <c r="A733" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B733" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C733" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D733" s="2" t="inlineStr">
+        <is>
+          <t>MTY81</t>
+        </is>
+      </c>
+      <c r="E733" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F733" s="3" t="n">
+        <v>288500</v>
+      </c>
+      <c r="G733" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="734">
+      <c r="A734" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B734" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C734" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D734" s="2" t="inlineStr">
+        <is>
+          <t>MTY87</t>
+        </is>
+      </c>
+      <c r="E734" s="2" t="inlineStr">
+        <is>
+          <t>Model Y L</t>
+        </is>
+      </c>
+      <c r="F734" s="3" t="n">
+        <v>339000</v>
+      </c>
+      <c r="G734" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="735">
+      <c r="A735" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B735" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C735" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D735" s="2" t="inlineStr">
+        <is>
+          <t>MTY88</t>
+        </is>
+      </c>
+      <c r="E735" s="2" t="inlineStr">
+        <is>
+          <t>Model Y Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F735" s="3" t="n">
+        <v>369000</v>
+      </c>
+      <c r="G735" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price pull 2026-10-19
</commit_message>
<xml_diff>
--- a/tesla_price_analysis.xlsx
+++ b/tesla_price_analysis.xlsx
@@ -445,7 +445,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Snapshot date: 2026-10-18  (source: tesla.com configurator pages)</t>
+          <t>Snapshot date: 2026-10-19  (source: tesla.com configurator pages)</t>
         </is>
       </c>
       <c r="B1" s="1" t="n"/>
@@ -997,7 +997,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G735"/>
+  <dimension ref="A1:G744"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -26736,6 +26736,321 @@
         </is>
       </c>
     </row>
+    <row r="736">
+      <c r="A736" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B736" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C736" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D736" s="2" t="inlineStr">
+        <is>
+          <t>MT380</t>
+        </is>
+      </c>
+      <c r="E736" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F736" s="3" t="n">
+        <v>339500</v>
+      </c>
+      <c r="G736" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="737">
+      <c r="A737" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B737" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C737" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D737" s="2" t="inlineStr">
+        <is>
+          <t>MT382</t>
+        </is>
+      </c>
+      <c r="E737" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F737" s="3" t="n">
+        <v>235500</v>
+      </c>
+      <c r="G737" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="738">
+      <c r="A738" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B738" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C738" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D738" s="2" t="inlineStr">
+        <is>
+          <t>MT383</t>
+        </is>
+      </c>
+      <c r="E738" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F738" s="3" t="n">
+        <v>259500</v>
+      </c>
+      <c r="G738" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="739">
+      <c r="A739" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B739" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C739" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D739" s="2" t="inlineStr">
+        <is>
+          <t>MT384</t>
+        </is>
+      </c>
+      <c r="E739" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F739" s="3" t="n">
+        <v>285500</v>
+      </c>
+      <c r="G739" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="740">
+      <c r="A740" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B740" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C740" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D740" s="2" t="inlineStr">
+        <is>
+          <t>MTY79</t>
+        </is>
+      </c>
+      <c r="E740" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F740" s="3" t="n">
+        <v>263500</v>
+      </c>
+      <c r="G740" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="741">
+      <c r="A741" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B741" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C741" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D741" s="2" t="inlineStr">
+        <is>
+          <t>MTY80</t>
+        </is>
+      </c>
+      <c r="E741" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F741" s="3" t="n">
+        <v>313500</v>
+      </c>
+      <c r="G741" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="742">
+      <c r="A742" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B742" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C742" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D742" s="2" t="inlineStr">
+        <is>
+          <t>MTY81</t>
+        </is>
+      </c>
+      <c r="E742" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F742" s="3" t="n">
+        <v>288500</v>
+      </c>
+      <c r="G742" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="743">
+      <c r="A743" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B743" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C743" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D743" s="2" t="inlineStr">
+        <is>
+          <t>MTY87</t>
+        </is>
+      </c>
+      <c r="E743" s="2" t="inlineStr">
+        <is>
+          <t>Model Y L</t>
+        </is>
+      </c>
+      <c r="F743" s="3" t="n">
+        <v>339000</v>
+      </c>
+      <c r="G743" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="744">
+      <c r="A744" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B744" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C744" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D744" s="2" t="inlineStr">
+        <is>
+          <t>MTY88</t>
+        </is>
+      </c>
+      <c r="E744" s="2" t="inlineStr">
+        <is>
+          <t>Model Y Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F744" s="3" t="n">
+        <v>369000</v>
+      </c>
+      <c r="G744" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price pull 2026-10-20
</commit_message>
<xml_diff>
--- a/tesla_price_analysis.xlsx
+++ b/tesla_price_analysis.xlsx
@@ -445,7 +445,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Snapshot date: 2026-10-19  (source: tesla.com configurator pages)</t>
+          <t>Snapshot date: 2026-10-20  (source: tesla.com configurator pages)</t>
         </is>
       </c>
       <c r="B1" s="1" t="n"/>
@@ -997,7 +997,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G744"/>
+  <dimension ref="A1:G753"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -27051,6 +27051,321 @@
         </is>
       </c>
     </row>
+    <row r="745">
+      <c r="A745" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B745" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C745" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D745" s="2" t="inlineStr">
+        <is>
+          <t>MT380</t>
+        </is>
+      </c>
+      <c r="E745" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F745" s="3" t="n">
+        <v>339500</v>
+      </c>
+      <c r="G745" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="746">
+      <c r="A746" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B746" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C746" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D746" s="2" t="inlineStr">
+        <is>
+          <t>MT382</t>
+        </is>
+      </c>
+      <c r="E746" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F746" s="3" t="n">
+        <v>235500</v>
+      </c>
+      <c r="G746" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="747">
+      <c r="A747" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B747" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C747" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D747" s="2" t="inlineStr">
+        <is>
+          <t>MT383</t>
+        </is>
+      </c>
+      <c r="E747" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F747" s="3" t="n">
+        <v>259500</v>
+      </c>
+      <c r="G747" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="748">
+      <c r="A748" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B748" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C748" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D748" s="2" t="inlineStr">
+        <is>
+          <t>MT384</t>
+        </is>
+      </c>
+      <c r="E748" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F748" s="3" t="n">
+        <v>285500</v>
+      </c>
+      <c r="G748" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="749">
+      <c r="A749" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B749" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C749" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D749" s="2" t="inlineStr">
+        <is>
+          <t>MTY79</t>
+        </is>
+      </c>
+      <c r="E749" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F749" s="3" t="n">
+        <v>263500</v>
+      </c>
+      <c r="G749" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="750">
+      <c r="A750" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B750" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C750" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D750" s="2" t="inlineStr">
+        <is>
+          <t>MTY80</t>
+        </is>
+      </c>
+      <c r="E750" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F750" s="3" t="n">
+        <v>313500</v>
+      </c>
+      <c r="G750" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="751">
+      <c r="A751" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B751" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C751" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D751" s="2" t="inlineStr">
+        <is>
+          <t>MTY81</t>
+        </is>
+      </c>
+      <c r="E751" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F751" s="3" t="n">
+        <v>288500</v>
+      </c>
+      <c r="G751" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="752">
+      <c r="A752" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B752" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C752" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D752" s="2" t="inlineStr">
+        <is>
+          <t>MTY87</t>
+        </is>
+      </c>
+      <c r="E752" s="2" t="inlineStr">
+        <is>
+          <t>Model Y L</t>
+        </is>
+      </c>
+      <c r="F752" s="3" t="n">
+        <v>339000</v>
+      </c>
+      <c r="G752" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="753">
+      <c r="A753" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="B753" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C753" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D753" s="2" t="inlineStr">
+        <is>
+          <t>MTY88</t>
+        </is>
+      </c>
+      <c r="E753" s="2" t="inlineStr">
+        <is>
+          <t>Model Y Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F753" s="3" t="n">
+        <v>369000</v>
+      </c>
+      <c r="G753" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price pull 2026-10-21
</commit_message>
<xml_diff>
--- a/tesla_price_analysis.xlsx
+++ b/tesla_price_analysis.xlsx
@@ -445,7 +445,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Snapshot date: 2026-10-20  (source: tesla.com configurator pages)</t>
+          <t>Snapshot date: 2026-10-21  (source: tesla.com configurator pages)</t>
         </is>
       </c>
       <c r="B1" s="1" t="n"/>
@@ -997,7 +997,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G753"/>
+  <dimension ref="A1:G762"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -27366,6 +27366,321 @@
         </is>
       </c>
     </row>
+    <row r="754">
+      <c r="A754" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B754" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C754" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D754" s="2" t="inlineStr">
+        <is>
+          <t>MT380</t>
+        </is>
+      </c>
+      <c r="E754" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F754" s="3" t="n">
+        <v>339500</v>
+      </c>
+      <c r="G754" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="755">
+      <c r="A755" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B755" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C755" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D755" s="2" t="inlineStr">
+        <is>
+          <t>MT382</t>
+        </is>
+      </c>
+      <c r="E755" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F755" s="3" t="n">
+        <v>235500</v>
+      </c>
+      <c r="G755" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="756">
+      <c r="A756" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B756" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C756" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D756" s="2" t="inlineStr">
+        <is>
+          <t>MT383</t>
+        </is>
+      </c>
+      <c r="E756" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F756" s="3" t="n">
+        <v>259500</v>
+      </c>
+      <c r="G756" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="757">
+      <c r="A757" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B757" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C757" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D757" s="2" t="inlineStr">
+        <is>
+          <t>MT384</t>
+        </is>
+      </c>
+      <c r="E757" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F757" s="3" t="n">
+        <v>285500</v>
+      </c>
+      <c r="G757" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="758">
+      <c r="A758" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B758" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C758" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D758" s="2" t="inlineStr">
+        <is>
+          <t>MTY79</t>
+        </is>
+      </c>
+      <c r="E758" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F758" s="3" t="n">
+        <v>263500</v>
+      </c>
+      <c r="G758" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="759">
+      <c r="A759" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B759" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C759" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D759" s="2" t="inlineStr">
+        <is>
+          <t>MTY80</t>
+        </is>
+      </c>
+      <c r="E759" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F759" s="3" t="n">
+        <v>313500</v>
+      </c>
+      <c r="G759" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="760">
+      <c r="A760" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B760" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C760" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D760" s="2" t="inlineStr">
+        <is>
+          <t>MTY81</t>
+        </is>
+      </c>
+      <c r="E760" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F760" s="3" t="n">
+        <v>288500</v>
+      </c>
+      <c r="G760" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="761">
+      <c r="A761" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B761" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C761" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D761" s="2" t="inlineStr">
+        <is>
+          <t>MTY87</t>
+        </is>
+      </c>
+      <c r="E761" s="2" t="inlineStr">
+        <is>
+          <t>Model Y L</t>
+        </is>
+      </c>
+      <c r="F761" s="3" t="n">
+        <v>339000</v>
+      </c>
+      <c r="G761" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="762">
+      <c r="A762" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="B762" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C762" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D762" s="2" t="inlineStr">
+        <is>
+          <t>MTY88</t>
+        </is>
+      </c>
+      <c r="E762" s="2" t="inlineStr">
+        <is>
+          <t>Model Y Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F762" s="3" t="n">
+        <v>369000</v>
+      </c>
+      <c r="G762" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price pull 2026-10-22
</commit_message>
<xml_diff>
--- a/tesla_price_analysis.xlsx
+++ b/tesla_price_analysis.xlsx
@@ -445,7 +445,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Snapshot date: 2026-10-21  (source: tesla.com configurator pages)</t>
+          <t>Snapshot date: 2026-10-22  (source: tesla.com configurator pages)</t>
         </is>
       </c>
       <c r="B1" s="1" t="n"/>
@@ -997,7 +997,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G762"/>
+  <dimension ref="A1:G771"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -27681,6 +27681,321 @@
         </is>
       </c>
     </row>
+    <row r="763">
+      <c r="A763" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B763" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C763" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D763" s="2" t="inlineStr">
+        <is>
+          <t>MT380</t>
+        </is>
+      </c>
+      <c r="E763" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F763" s="3" t="n">
+        <v>339500</v>
+      </c>
+      <c r="G763" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="764">
+      <c r="A764" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B764" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C764" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D764" s="2" t="inlineStr">
+        <is>
+          <t>MT382</t>
+        </is>
+      </c>
+      <c r="E764" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F764" s="3" t="n">
+        <v>235500</v>
+      </c>
+      <c r="G764" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="765">
+      <c r="A765" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B765" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C765" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D765" s="2" t="inlineStr">
+        <is>
+          <t>MT383</t>
+        </is>
+      </c>
+      <c r="E765" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F765" s="3" t="n">
+        <v>259500</v>
+      </c>
+      <c r="G765" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="766">
+      <c r="A766" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B766" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C766" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D766" s="2" t="inlineStr">
+        <is>
+          <t>MT384</t>
+        </is>
+      </c>
+      <c r="E766" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F766" s="3" t="n">
+        <v>285500</v>
+      </c>
+      <c r="G766" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="767">
+      <c r="A767" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B767" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C767" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D767" s="2" t="inlineStr">
+        <is>
+          <t>MTY79</t>
+        </is>
+      </c>
+      <c r="E767" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F767" s="3" t="n">
+        <v>263500</v>
+      </c>
+      <c r="G767" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="768">
+      <c r="A768" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B768" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C768" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D768" s="2" t="inlineStr">
+        <is>
+          <t>MTY80</t>
+        </is>
+      </c>
+      <c r="E768" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F768" s="3" t="n">
+        <v>313500</v>
+      </c>
+      <c r="G768" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="769">
+      <c r="A769" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B769" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C769" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D769" s="2" t="inlineStr">
+        <is>
+          <t>MTY81</t>
+        </is>
+      </c>
+      <c r="E769" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F769" s="3" t="n">
+        <v>288500</v>
+      </c>
+      <c r="G769" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="770">
+      <c r="A770" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B770" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C770" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D770" s="2" t="inlineStr">
+        <is>
+          <t>MTY87</t>
+        </is>
+      </c>
+      <c r="E770" s="2" t="inlineStr">
+        <is>
+          <t>Model Y L</t>
+        </is>
+      </c>
+      <c r="F770" s="3" t="n">
+        <v>339000</v>
+      </c>
+      <c r="G770" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="771">
+      <c r="A771" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="B771" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C771" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D771" s="2" t="inlineStr">
+        <is>
+          <t>MTY88</t>
+        </is>
+      </c>
+      <c r="E771" s="2" t="inlineStr">
+        <is>
+          <t>Model Y Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F771" s="3" t="n">
+        <v>369000</v>
+      </c>
+      <c r="G771" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price pull 2026-10-23
</commit_message>
<xml_diff>
--- a/tesla_price_analysis.xlsx
+++ b/tesla_price_analysis.xlsx
@@ -445,7 +445,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Snapshot date: 2026-10-22  (source: tesla.com configurator pages)</t>
+          <t>Snapshot date: 2026-10-23  (source: tesla.com configurator pages)</t>
         </is>
       </c>
       <c r="B1" s="1" t="n"/>
@@ -997,7 +997,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G771"/>
+  <dimension ref="A1:G780"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -27996,6 +27996,321 @@
         </is>
       </c>
     </row>
+    <row r="772">
+      <c r="A772" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B772" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C772" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D772" s="2" t="inlineStr">
+        <is>
+          <t>MT380</t>
+        </is>
+      </c>
+      <c r="E772" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F772" s="3" t="n">
+        <v>339500</v>
+      </c>
+      <c r="G772" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="773">
+      <c r="A773" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B773" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C773" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D773" s="2" t="inlineStr">
+        <is>
+          <t>MT382</t>
+        </is>
+      </c>
+      <c r="E773" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F773" s="3" t="n">
+        <v>235500</v>
+      </c>
+      <c r="G773" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="774">
+      <c r="A774" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B774" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C774" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D774" s="2" t="inlineStr">
+        <is>
+          <t>MT383</t>
+        </is>
+      </c>
+      <c r="E774" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F774" s="3" t="n">
+        <v>259500</v>
+      </c>
+      <c r="G774" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="775">
+      <c r="A775" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B775" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C775" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D775" s="2" t="inlineStr">
+        <is>
+          <t>MT384</t>
+        </is>
+      </c>
+      <c r="E775" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F775" s="3" t="n">
+        <v>285500</v>
+      </c>
+      <c r="G775" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="776">
+      <c r="A776" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B776" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C776" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D776" s="2" t="inlineStr">
+        <is>
+          <t>MTY79</t>
+        </is>
+      </c>
+      <c r="E776" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F776" s="3" t="n">
+        <v>263500</v>
+      </c>
+      <c r="G776" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="777">
+      <c r="A777" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B777" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C777" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D777" s="2" t="inlineStr">
+        <is>
+          <t>MTY80</t>
+        </is>
+      </c>
+      <c r="E777" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F777" s="3" t="n">
+        <v>313500</v>
+      </c>
+      <c r="G777" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="778">
+      <c r="A778" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B778" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C778" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D778" s="2" t="inlineStr">
+        <is>
+          <t>MTY81</t>
+        </is>
+      </c>
+      <c r="E778" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F778" s="3" t="n">
+        <v>288500</v>
+      </c>
+      <c r="G778" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="779">
+      <c r="A779" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B779" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C779" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D779" s="2" t="inlineStr">
+        <is>
+          <t>MTY87</t>
+        </is>
+      </c>
+      <c r="E779" s="2" t="inlineStr">
+        <is>
+          <t>Model Y L</t>
+        </is>
+      </c>
+      <c r="F779" s="3" t="n">
+        <v>339000</v>
+      </c>
+      <c r="G779" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="780">
+      <c r="A780" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B780" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C780" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D780" s="2" t="inlineStr">
+        <is>
+          <t>MTY88</t>
+        </is>
+      </c>
+      <c r="E780" s="2" t="inlineStr">
+        <is>
+          <t>Model Y Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F780" s="3" t="n">
+        <v>369000</v>
+      </c>
+      <c r="G780" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price pull 2026-10-24
</commit_message>
<xml_diff>
--- a/tesla_price_analysis.xlsx
+++ b/tesla_price_analysis.xlsx
@@ -445,7 +445,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Snapshot date: 2026-10-23  (source: tesla.com configurator pages)</t>
+          <t>Snapshot date: 2026-10-24  (source: tesla.com configurator pages)</t>
         </is>
       </c>
       <c r="B1" s="1" t="n"/>
@@ -997,7 +997,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G780"/>
+  <dimension ref="A1:G789"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -28311,6 +28311,321 @@
         </is>
       </c>
     </row>
+    <row r="781">
+      <c r="A781" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B781" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C781" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D781" s="2" t="inlineStr">
+        <is>
+          <t>MT380</t>
+        </is>
+      </c>
+      <c r="E781" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F781" s="3" t="n">
+        <v>339500</v>
+      </c>
+      <c r="G781" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="782">
+      <c r="A782" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B782" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C782" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D782" s="2" t="inlineStr">
+        <is>
+          <t>MT382</t>
+        </is>
+      </c>
+      <c r="E782" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F782" s="3" t="n">
+        <v>235500</v>
+      </c>
+      <c r="G782" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="783">
+      <c r="A783" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B783" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C783" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D783" s="2" t="inlineStr">
+        <is>
+          <t>MT383</t>
+        </is>
+      </c>
+      <c r="E783" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F783" s="3" t="n">
+        <v>259500</v>
+      </c>
+      <c r="G783" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="784">
+      <c r="A784" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B784" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C784" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D784" s="2" t="inlineStr">
+        <is>
+          <t>MT384</t>
+        </is>
+      </c>
+      <c r="E784" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F784" s="3" t="n">
+        <v>285500</v>
+      </c>
+      <c r="G784" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="785">
+      <c r="A785" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B785" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C785" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D785" s="2" t="inlineStr">
+        <is>
+          <t>MTY79</t>
+        </is>
+      </c>
+      <c r="E785" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F785" s="3" t="n">
+        <v>263500</v>
+      </c>
+      <c r="G785" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="786">
+      <c r="A786" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B786" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C786" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D786" s="2" t="inlineStr">
+        <is>
+          <t>MTY80</t>
+        </is>
+      </c>
+      <c r="E786" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F786" s="3" t="n">
+        <v>313500</v>
+      </c>
+      <c r="G786" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="787">
+      <c r="A787" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B787" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C787" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D787" s="2" t="inlineStr">
+        <is>
+          <t>MTY81</t>
+        </is>
+      </c>
+      <c r="E787" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F787" s="3" t="n">
+        <v>288500</v>
+      </c>
+      <c r="G787" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="788">
+      <c r="A788" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B788" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C788" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D788" s="2" t="inlineStr">
+        <is>
+          <t>MTY87</t>
+        </is>
+      </c>
+      <c r="E788" s="2" t="inlineStr">
+        <is>
+          <t>Model Y L</t>
+        </is>
+      </c>
+      <c r="F788" s="3" t="n">
+        <v>339000</v>
+      </c>
+      <c r="G788" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="789">
+      <c r="A789" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B789" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C789" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D789" s="2" t="inlineStr">
+        <is>
+          <t>MTY88</t>
+        </is>
+      </c>
+      <c r="E789" s="2" t="inlineStr">
+        <is>
+          <t>Model Y Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F789" s="3" t="n">
+        <v>369000</v>
+      </c>
+      <c r="G789" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price pull 2026-10-25
</commit_message>
<xml_diff>
--- a/tesla_price_analysis.xlsx
+++ b/tesla_price_analysis.xlsx
@@ -445,7 +445,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Snapshot date: 2026-10-24  (source: tesla.com configurator pages)</t>
+          <t>Snapshot date: 2026-10-25  (source: tesla.com configurator pages)</t>
         </is>
       </c>
       <c r="B1" s="1" t="n"/>
@@ -997,7 +997,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G789"/>
+  <dimension ref="A1:G798"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -28626,6 +28626,321 @@
         </is>
       </c>
     </row>
+    <row r="790">
+      <c r="A790" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B790" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C790" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D790" s="2" t="inlineStr">
+        <is>
+          <t>MT380</t>
+        </is>
+      </c>
+      <c r="E790" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F790" s="3" t="n">
+        <v>339500</v>
+      </c>
+      <c r="G790" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="791">
+      <c r="A791" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B791" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C791" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D791" s="2" t="inlineStr">
+        <is>
+          <t>MT382</t>
+        </is>
+      </c>
+      <c r="E791" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F791" s="3" t="n">
+        <v>235500</v>
+      </c>
+      <c r="G791" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="792">
+      <c r="A792" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B792" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C792" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D792" s="2" t="inlineStr">
+        <is>
+          <t>MT383</t>
+        </is>
+      </c>
+      <c r="E792" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F792" s="3" t="n">
+        <v>259500</v>
+      </c>
+      <c r="G792" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="793">
+      <c r="A793" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B793" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C793" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D793" s="2" t="inlineStr">
+        <is>
+          <t>MT384</t>
+        </is>
+      </c>
+      <c r="E793" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F793" s="3" t="n">
+        <v>285500</v>
+      </c>
+      <c r="G793" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="794">
+      <c r="A794" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B794" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C794" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D794" s="2" t="inlineStr">
+        <is>
+          <t>MTY79</t>
+        </is>
+      </c>
+      <c r="E794" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F794" s="3" t="n">
+        <v>263500</v>
+      </c>
+      <c r="G794" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="795">
+      <c r="A795" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B795" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C795" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D795" s="2" t="inlineStr">
+        <is>
+          <t>MTY80</t>
+        </is>
+      </c>
+      <c r="E795" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F795" s="3" t="n">
+        <v>313500</v>
+      </c>
+      <c r="G795" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="796">
+      <c r="A796" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B796" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C796" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D796" s="2" t="inlineStr">
+        <is>
+          <t>MTY81</t>
+        </is>
+      </c>
+      <c r="E796" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F796" s="3" t="n">
+        <v>288500</v>
+      </c>
+      <c r="G796" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="797">
+      <c r="A797" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B797" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C797" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D797" s="2" t="inlineStr">
+        <is>
+          <t>MTY87</t>
+        </is>
+      </c>
+      <c r="E797" s="2" t="inlineStr">
+        <is>
+          <t>Model Y L</t>
+        </is>
+      </c>
+      <c r="F797" s="3" t="n">
+        <v>339000</v>
+      </c>
+      <c r="G797" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="798">
+      <c r="A798" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B798" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C798" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D798" s="2" t="inlineStr">
+        <is>
+          <t>MTY88</t>
+        </is>
+      </c>
+      <c r="E798" s="2" t="inlineStr">
+        <is>
+          <t>Model Y Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F798" s="3" t="n">
+        <v>369000</v>
+      </c>
+      <c r="G798" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price pull 2026-10-26
</commit_message>
<xml_diff>
--- a/tesla_price_analysis.xlsx
+++ b/tesla_price_analysis.xlsx
@@ -445,7 +445,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Snapshot date: 2026-10-25  (source: tesla.com configurator pages)</t>
+          <t>Snapshot date: 2026-10-26  (source: tesla.com configurator pages)</t>
         </is>
       </c>
       <c r="B1" s="1" t="n"/>
@@ -997,7 +997,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G798"/>
+  <dimension ref="A1:G807"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -28941,6 +28941,321 @@
         </is>
       </c>
     </row>
+    <row r="799">
+      <c r="A799" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B799" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C799" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D799" s="2" t="inlineStr">
+        <is>
+          <t>MT380</t>
+        </is>
+      </c>
+      <c r="E799" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F799" s="3" t="n">
+        <v>339500</v>
+      </c>
+      <c r="G799" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="800">
+      <c r="A800" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B800" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C800" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D800" s="2" t="inlineStr">
+        <is>
+          <t>MT382</t>
+        </is>
+      </c>
+      <c r="E800" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F800" s="3" t="n">
+        <v>235500</v>
+      </c>
+      <c r="G800" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="801">
+      <c r="A801" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B801" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C801" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D801" s="2" t="inlineStr">
+        <is>
+          <t>MT383</t>
+        </is>
+      </c>
+      <c r="E801" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F801" s="3" t="n">
+        <v>259500</v>
+      </c>
+      <c r="G801" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="802">
+      <c r="A802" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B802" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C802" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D802" s="2" t="inlineStr">
+        <is>
+          <t>MT384</t>
+        </is>
+      </c>
+      <c r="E802" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F802" s="3" t="n">
+        <v>285500</v>
+      </c>
+      <c r="G802" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="803">
+      <c r="A803" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B803" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C803" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D803" s="2" t="inlineStr">
+        <is>
+          <t>MTY79</t>
+        </is>
+      </c>
+      <c r="E803" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F803" s="3" t="n">
+        <v>263500</v>
+      </c>
+      <c r="G803" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="804">
+      <c r="A804" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B804" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C804" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D804" s="2" t="inlineStr">
+        <is>
+          <t>MTY80</t>
+        </is>
+      </c>
+      <c r="E804" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F804" s="3" t="n">
+        <v>313500</v>
+      </c>
+      <c r="G804" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="805">
+      <c r="A805" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B805" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C805" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D805" s="2" t="inlineStr">
+        <is>
+          <t>MTY81</t>
+        </is>
+      </c>
+      <c r="E805" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F805" s="3" t="n">
+        <v>288500</v>
+      </c>
+      <c r="G805" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="806">
+      <c r="A806" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B806" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C806" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D806" s="2" t="inlineStr">
+        <is>
+          <t>MTY87</t>
+        </is>
+      </c>
+      <c r="E806" s="2" t="inlineStr">
+        <is>
+          <t>Model Y L</t>
+        </is>
+      </c>
+      <c r="F806" s="3" t="n">
+        <v>339000</v>
+      </c>
+      <c r="G806" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="807">
+      <c r="A807" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B807" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C807" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D807" s="2" t="inlineStr">
+        <is>
+          <t>MTY88</t>
+        </is>
+      </c>
+      <c r="E807" s="2" t="inlineStr">
+        <is>
+          <t>Model Y Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F807" s="3" t="n">
+        <v>369000</v>
+      </c>
+      <c r="G807" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price pull 2026-10-27
</commit_message>
<xml_diff>
--- a/tesla_price_analysis.xlsx
+++ b/tesla_price_analysis.xlsx
@@ -445,7 +445,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Snapshot date: 2026-10-26  (source: tesla.com configurator pages)</t>
+          <t>Snapshot date: 2026-10-27  (source: tesla.com configurator pages)</t>
         </is>
       </c>
       <c r="B1" s="1" t="n"/>
@@ -997,7 +997,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G807"/>
+  <dimension ref="A1:G816"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -29256,6 +29256,321 @@
         </is>
       </c>
     </row>
+    <row r="808">
+      <c r="A808" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B808" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C808" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D808" s="2" t="inlineStr">
+        <is>
+          <t>MT380</t>
+        </is>
+      </c>
+      <c r="E808" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F808" s="3" t="n">
+        <v>339500</v>
+      </c>
+      <c r="G808" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="809">
+      <c r="A809" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B809" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C809" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D809" s="2" t="inlineStr">
+        <is>
+          <t>MT382</t>
+        </is>
+      </c>
+      <c r="E809" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F809" s="3" t="n">
+        <v>235500</v>
+      </c>
+      <c r="G809" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="810">
+      <c r="A810" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B810" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C810" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D810" s="2" t="inlineStr">
+        <is>
+          <t>MT383</t>
+        </is>
+      </c>
+      <c r="E810" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F810" s="3" t="n">
+        <v>259500</v>
+      </c>
+      <c r="G810" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="811">
+      <c r="A811" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B811" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C811" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D811" s="2" t="inlineStr">
+        <is>
+          <t>MT384</t>
+        </is>
+      </c>
+      <c r="E811" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F811" s="3" t="n">
+        <v>285500</v>
+      </c>
+      <c r="G811" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="812">
+      <c r="A812" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B812" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C812" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D812" s="2" t="inlineStr">
+        <is>
+          <t>MTY79</t>
+        </is>
+      </c>
+      <c r="E812" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F812" s="3" t="n">
+        <v>263500</v>
+      </c>
+      <c r="G812" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="813">
+      <c r="A813" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B813" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C813" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D813" s="2" t="inlineStr">
+        <is>
+          <t>MTY80</t>
+        </is>
+      </c>
+      <c r="E813" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F813" s="3" t="n">
+        <v>313500</v>
+      </c>
+      <c r="G813" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="814">
+      <c r="A814" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B814" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C814" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D814" s="2" t="inlineStr">
+        <is>
+          <t>MTY81</t>
+        </is>
+      </c>
+      <c r="E814" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F814" s="3" t="n">
+        <v>288500</v>
+      </c>
+      <c r="G814" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="815">
+      <c r="A815" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B815" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C815" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D815" s="2" t="inlineStr">
+        <is>
+          <t>MTY87</t>
+        </is>
+      </c>
+      <c r="E815" s="2" t="inlineStr">
+        <is>
+          <t>Model Y L</t>
+        </is>
+      </c>
+      <c r="F815" s="3" t="n">
+        <v>339000</v>
+      </c>
+      <c r="G815" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="816">
+      <c r="A816" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B816" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C816" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D816" s="2" t="inlineStr">
+        <is>
+          <t>MTY88</t>
+        </is>
+      </c>
+      <c r="E816" s="2" t="inlineStr">
+        <is>
+          <t>Model Y Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F816" s="3" t="n">
+        <v>369000</v>
+      </c>
+      <c r="G816" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price pull 2026-10-28
</commit_message>
<xml_diff>
--- a/tesla_price_analysis.xlsx
+++ b/tesla_price_analysis.xlsx
@@ -445,7 +445,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Snapshot date: 2026-10-27  (source: tesla.com configurator pages)</t>
+          <t>Snapshot date: 2026-10-28  (source: tesla.com configurator pages)</t>
         </is>
       </c>
       <c r="B1" s="1" t="n"/>
@@ -997,7 +997,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G816"/>
+  <dimension ref="A1:G825"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -29571,6 +29571,321 @@
         </is>
       </c>
     </row>
+    <row r="817">
+      <c r="A817" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B817" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C817" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D817" s="2" t="inlineStr">
+        <is>
+          <t>MT380</t>
+        </is>
+      </c>
+      <c r="E817" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F817" s="3" t="n">
+        <v>339500</v>
+      </c>
+      <c r="G817" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="818">
+      <c r="A818" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B818" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C818" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D818" s="2" t="inlineStr">
+        <is>
+          <t>MT382</t>
+        </is>
+      </c>
+      <c r="E818" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F818" s="3" t="n">
+        <v>235500</v>
+      </c>
+      <c r="G818" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="819">
+      <c r="A819" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B819" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C819" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D819" s="2" t="inlineStr">
+        <is>
+          <t>MT383</t>
+        </is>
+      </c>
+      <c r="E819" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F819" s="3" t="n">
+        <v>259500</v>
+      </c>
+      <c r="G819" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="820">
+      <c r="A820" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B820" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C820" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D820" s="2" t="inlineStr">
+        <is>
+          <t>MT384</t>
+        </is>
+      </c>
+      <c r="E820" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F820" s="3" t="n">
+        <v>285500</v>
+      </c>
+      <c r="G820" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="821">
+      <c r="A821" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B821" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C821" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D821" s="2" t="inlineStr">
+        <is>
+          <t>MTY79</t>
+        </is>
+      </c>
+      <c r="E821" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F821" s="3" t="n">
+        <v>263500</v>
+      </c>
+      <c r="G821" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="822">
+      <c r="A822" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B822" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C822" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D822" s="2" t="inlineStr">
+        <is>
+          <t>MTY80</t>
+        </is>
+      </c>
+      <c r="E822" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F822" s="3" t="n">
+        <v>313500</v>
+      </c>
+      <c r="G822" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="823">
+      <c r="A823" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B823" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C823" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D823" s="2" t="inlineStr">
+        <is>
+          <t>MTY81</t>
+        </is>
+      </c>
+      <c r="E823" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F823" s="3" t="n">
+        <v>288500</v>
+      </c>
+      <c r="G823" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="824">
+      <c r="A824" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B824" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C824" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D824" s="2" t="inlineStr">
+        <is>
+          <t>MTY87</t>
+        </is>
+      </c>
+      <c r="E824" s="2" t="inlineStr">
+        <is>
+          <t>Model Y L</t>
+        </is>
+      </c>
+      <c r="F824" s="3" t="n">
+        <v>339000</v>
+      </c>
+      <c r="G824" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="825">
+      <c r="A825" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B825" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C825" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D825" s="2" t="inlineStr">
+        <is>
+          <t>MTY88</t>
+        </is>
+      </c>
+      <c r="E825" s="2" t="inlineStr">
+        <is>
+          <t>Model Y Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F825" s="3" t="n">
+        <v>369000</v>
+      </c>
+      <c r="G825" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price pull 2026-10-29
</commit_message>
<xml_diff>
--- a/tesla_price_analysis.xlsx
+++ b/tesla_price_analysis.xlsx
@@ -445,7 +445,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Snapshot date: 2026-10-28  (source: tesla.com configurator pages)</t>
+          <t>Snapshot date: 2026-10-29  (source: tesla.com configurator pages)</t>
         </is>
       </c>
       <c r="B1" s="1" t="n"/>
@@ -997,7 +997,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G825"/>
+  <dimension ref="A1:G834"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -29886,6 +29886,321 @@
         </is>
       </c>
     </row>
+    <row r="826">
+      <c r="A826" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B826" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C826" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D826" s="2" t="inlineStr">
+        <is>
+          <t>MT380</t>
+        </is>
+      </c>
+      <c r="E826" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F826" s="3" t="n">
+        <v>339500</v>
+      </c>
+      <c r="G826" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="827">
+      <c r="A827" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B827" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C827" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D827" s="2" t="inlineStr">
+        <is>
+          <t>MT382</t>
+        </is>
+      </c>
+      <c r="E827" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F827" s="3" t="n">
+        <v>235500</v>
+      </c>
+      <c r="G827" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="828">
+      <c r="A828" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B828" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C828" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D828" s="2" t="inlineStr">
+        <is>
+          <t>MT383</t>
+        </is>
+      </c>
+      <c r="E828" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F828" s="3" t="n">
+        <v>259500</v>
+      </c>
+      <c r="G828" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="829">
+      <c r="A829" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B829" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C829" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D829" s="2" t="inlineStr">
+        <is>
+          <t>MT384</t>
+        </is>
+      </c>
+      <c r="E829" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F829" s="3" t="n">
+        <v>285500</v>
+      </c>
+      <c r="G829" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="830">
+      <c r="A830" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B830" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C830" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D830" s="2" t="inlineStr">
+        <is>
+          <t>MTY79</t>
+        </is>
+      </c>
+      <c r="E830" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F830" s="3" t="n">
+        <v>263500</v>
+      </c>
+      <c r="G830" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="831">
+      <c r="A831" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B831" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C831" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D831" s="2" t="inlineStr">
+        <is>
+          <t>MTY80</t>
+        </is>
+      </c>
+      <c r="E831" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F831" s="3" t="n">
+        <v>313500</v>
+      </c>
+      <c r="G831" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="832">
+      <c r="A832" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B832" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C832" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D832" s="2" t="inlineStr">
+        <is>
+          <t>MTY81</t>
+        </is>
+      </c>
+      <c r="E832" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F832" s="3" t="n">
+        <v>288500</v>
+      </c>
+      <c r="G832" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="833">
+      <c r="A833" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B833" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C833" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D833" s="2" t="inlineStr">
+        <is>
+          <t>MTY87</t>
+        </is>
+      </c>
+      <c r="E833" s="2" t="inlineStr">
+        <is>
+          <t>Model Y L</t>
+        </is>
+      </c>
+      <c r="F833" s="3" t="n">
+        <v>339000</v>
+      </c>
+      <c r="G833" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="834">
+      <c r="A834" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B834" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C834" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D834" s="2" t="inlineStr">
+        <is>
+          <t>MTY88</t>
+        </is>
+      </c>
+      <c r="E834" s="2" t="inlineStr">
+        <is>
+          <t>Model Y Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F834" s="3" t="n">
+        <v>369000</v>
+      </c>
+      <c r="G834" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price pull 2026-10-30
</commit_message>
<xml_diff>
--- a/tesla_price_analysis.xlsx
+++ b/tesla_price_analysis.xlsx
@@ -445,7 +445,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Snapshot date: 2026-10-29  (source: tesla.com configurator pages)</t>
+          <t>Snapshot date: 2026-10-30  (source: tesla.com configurator pages)</t>
         </is>
       </c>
       <c r="B1" s="1" t="n"/>
@@ -997,7 +997,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G834"/>
+  <dimension ref="A1:G843"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -30201,6 +30201,321 @@
         </is>
       </c>
     </row>
+    <row r="835">
+      <c r="A835" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B835" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C835" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D835" s="2" t="inlineStr">
+        <is>
+          <t>MT380</t>
+        </is>
+      </c>
+      <c r="E835" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F835" s="3" t="n">
+        <v>339500</v>
+      </c>
+      <c r="G835" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="836">
+      <c r="A836" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B836" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C836" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D836" s="2" t="inlineStr">
+        <is>
+          <t>MT382</t>
+        </is>
+      </c>
+      <c r="E836" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F836" s="3" t="n">
+        <v>235500</v>
+      </c>
+      <c r="G836" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="837">
+      <c r="A837" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B837" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C837" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D837" s="2" t="inlineStr">
+        <is>
+          <t>MT383</t>
+        </is>
+      </c>
+      <c r="E837" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F837" s="3" t="n">
+        <v>259500</v>
+      </c>
+      <c r="G837" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="838">
+      <c r="A838" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B838" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C838" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D838" s="2" t="inlineStr">
+        <is>
+          <t>MT384</t>
+        </is>
+      </c>
+      <c r="E838" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F838" s="3" t="n">
+        <v>285500</v>
+      </c>
+      <c r="G838" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="839">
+      <c r="A839" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B839" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C839" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D839" s="2" t="inlineStr">
+        <is>
+          <t>MTY79</t>
+        </is>
+      </c>
+      <c r="E839" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F839" s="3" t="n">
+        <v>263500</v>
+      </c>
+      <c r="G839" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="840">
+      <c r="A840" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B840" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C840" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D840" s="2" t="inlineStr">
+        <is>
+          <t>MTY80</t>
+        </is>
+      </c>
+      <c r="E840" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F840" s="3" t="n">
+        <v>313500</v>
+      </c>
+      <c r="G840" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="841">
+      <c r="A841" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B841" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C841" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D841" s="2" t="inlineStr">
+        <is>
+          <t>MTY81</t>
+        </is>
+      </c>
+      <c r="E841" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F841" s="3" t="n">
+        <v>288500</v>
+      </c>
+      <c r="G841" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="842">
+      <c r="A842" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B842" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C842" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D842" s="2" t="inlineStr">
+        <is>
+          <t>MTY87</t>
+        </is>
+      </c>
+      <c r="E842" s="2" t="inlineStr">
+        <is>
+          <t>Model Y L</t>
+        </is>
+      </c>
+      <c r="F842" s="3" t="n">
+        <v>339000</v>
+      </c>
+      <c r="G842" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="843">
+      <c r="A843" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B843" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C843" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D843" s="2" t="inlineStr">
+        <is>
+          <t>MTY88</t>
+        </is>
+      </c>
+      <c r="E843" s="2" t="inlineStr">
+        <is>
+          <t>Model Y Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F843" s="3" t="n">
+        <v>369000</v>
+      </c>
+      <c r="G843" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price pull 2026-10-31
</commit_message>
<xml_diff>
--- a/tesla_price_analysis.xlsx
+++ b/tesla_price_analysis.xlsx
@@ -445,7 +445,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Snapshot date: 2026-10-30  (source: tesla.com configurator pages)</t>
+          <t>Snapshot date: 2026-10-31  (source: tesla.com configurator pages)</t>
         </is>
       </c>
       <c r="B1" s="1" t="n"/>
@@ -997,7 +997,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G843"/>
+  <dimension ref="A1:G852"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -30516,6 +30516,321 @@
         </is>
       </c>
     </row>
+    <row r="844">
+      <c r="A844" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="B844" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C844" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D844" s="2" t="inlineStr">
+        <is>
+          <t>MT380</t>
+        </is>
+      </c>
+      <c r="E844" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F844" s="3" t="n">
+        <v>339500</v>
+      </c>
+      <c r="G844" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="845">
+      <c r="A845" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="B845" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C845" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D845" s="2" t="inlineStr">
+        <is>
+          <t>MT382</t>
+        </is>
+      </c>
+      <c r="E845" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F845" s="3" t="n">
+        <v>235500</v>
+      </c>
+      <c r="G845" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="846">
+      <c r="A846" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="B846" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C846" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D846" s="2" t="inlineStr">
+        <is>
+          <t>MT383</t>
+        </is>
+      </c>
+      <c r="E846" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F846" s="3" t="n">
+        <v>259500</v>
+      </c>
+      <c r="G846" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="847">
+      <c r="A847" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="B847" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C847" s="2" t="inlineStr">
+        <is>
+          <t>model3</t>
+        </is>
+      </c>
+      <c r="D847" s="2" t="inlineStr">
+        <is>
+          <t>MT384</t>
+        </is>
+      </c>
+      <c r="E847" s="2" t="inlineStr">
+        <is>
+          <t>Model 3 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F847" s="3" t="n">
+        <v>285500</v>
+      </c>
+      <c r="G847" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="848">
+      <c r="A848" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="B848" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C848" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D848" s="2" t="inlineStr">
+        <is>
+          <t>MTY79</t>
+        </is>
+      </c>
+      <c r="E848" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F848" s="3" t="n">
+        <v>263500</v>
+      </c>
+      <c r="G848" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="849">
+      <c r="A849" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="B849" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C849" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D849" s="2" t="inlineStr">
+        <is>
+          <t>MTY80</t>
+        </is>
+      </c>
+      <c r="E849" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F849" s="3" t="n">
+        <v>313500</v>
+      </c>
+      <c r="G849" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="850">
+      <c r="A850" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="B850" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C850" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D850" s="2" t="inlineStr">
+        <is>
+          <t>MTY81</t>
+        </is>
+      </c>
+      <c r="E850" s="2" t="inlineStr">
+        <is>
+          <t>Model Y 长续航后轮驱动版</t>
+        </is>
+      </c>
+      <c r="F850" s="3" t="n">
+        <v>288500</v>
+      </c>
+      <c r="G850" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="851">
+      <c r="A851" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="B851" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C851" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D851" s="2" t="inlineStr">
+        <is>
+          <t>MTY87</t>
+        </is>
+      </c>
+      <c r="E851" s="2" t="inlineStr">
+        <is>
+          <t>Model Y L</t>
+        </is>
+      </c>
+      <c r="F851" s="3" t="n">
+        <v>339000</v>
+      </c>
+      <c r="G851" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="852">
+      <c r="A852" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="B852" s="2" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="C852" s="2" t="inlineStr">
+        <is>
+          <t>modely</t>
+        </is>
+      </c>
+      <c r="D852" s="2" t="inlineStr">
+        <is>
+          <t>MTY88</t>
+        </is>
+      </c>
+      <c r="E852" s="2" t="inlineStr">
+        <is>
+          <t>Model Y Performance 高性能全轮驱动版</t>
+        </is>
+      </c>
+      <c r="F852" s="3" t="n">
+        <v>369000</v>
+      </c>
+      <c r="G852" s="2" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>